<commit_message>
Acama on its $22.07M GMP in all plans and the FY2027 budget; agenda in Pacific; safety reads no recordable incidents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EkVDtrr64Hp1gx17meyeHf
</commit_message>
<xml_diff>
--- a/models/SixPeak_OperatingBudget_2026-10-28.xlsx
+++ b/models/SixPeak_OperatingBudget_2026-10-28.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="361">
   <si>
     <t xml:space="preserve">Six Peak consolidated FY2027 budget</t>
   </si>
@@ -172,7 +172,7 @@
     <t xml:space="preserve">Closing cash</t>
   </si>
   <si>
-    <t xml:space="preserve">Opening cash is the model's 31 Dec 2026 balance (from the 30 Sep 2026 ledger), with Acama's $536K Krueger fee held to January. Developer fees to Six Peak and APA are received as earned.</t>
+    <t xml:space="preserve">Opening cash is the model's 31 Dec 2026 balance (from the 30 Sep 2026 ledger). Acama's $561,958 Krueger fee is held to January; developer fees to Six Peak and APA are received as earned.</t>
   </si>
   <si>
     <t xml:space="preserve">MEMO</t>
@@ -1030,13 +1030,13 @@
     <t xml:space="preserve">Model columns N:Y = Jan-Dec 2027; values frozen, totals are formulas</t>
   </si>
   <si>
-    <t xml:space="preserve">Check: LV NI. Base Case Model row 237, FY2027 (models _2026-10-28; the model carries the pay-app automation since 26 Oct). Should equal Consolidated!N23.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check: Six Peak NI. Base Case Model row 293 FY2027. Should equal Consolidated!N24.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Older check values (LV 4,297,655 and consolidated 2,299,779) were pre-adjustment figures from the 20 Oct build; replaced 28 Oct with the checks above, which tie to this budget.</t>
+    <t xml:space="preserve">Check: LV NI. Base Case Model row 237, FY2027 (models _2026-10-28). Should equal Consolidated!N23.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check: Six Peak NI. Base Case Model row 293, FY2027. Should equal Consolidated!N24.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Older check values (LV 4,297,655 and consolidated 2,299,779) were pre-adjustment figures from the 20 Oct build; replaced 28 Oct with checks that tie to this budget.</t>
   </si>
   <si>
     <t xml:space="preserve">Check: APA NI = APA Inc. FY2027 budget file, row 65 (replaces Model row 297)</t>
@@ -1099,13 +1099,16 @@
     <t xml:space="preserve">What-moves-it figures rerun 26 Oct 2026 on the final Base Case (models _2026-10-26): Reseda off -320,878; Beverly off -97,401; Acama at the Dec 2026 start +409,364 (so the slip costs 409,364).</t>
   </si>
   <si>
-    <t xml:space="preserve">28 Oct 2026 (Chris): (1) Superintendent rate corrected. Staffing engine superintendent slots 6-10 were priced at the assistant superintendent rate ($125,000); now $160,000 like slots 1-5. Affects the October 2027 superintendent (Kester, Beverly): LV payroll and burden plus placement fee -12,364 in FY2027. (2) Acama bond actuals: bond issued 12 Oct 2026 on the $22,072,845 GMP; bond line $326,200 (invoice LV-2026-ACA-01), CBI premium $155,409 (invoice #024003), Krueger cash $561,958 (615 Holdings schedule 28 Oct). Bond month Oct 2026 (was Dec 2026). FY2026 NI -14,345; Krueger January payout 1,228,421 -&gt; 1,254,835; tax distribution 245,851 -&gt; 238,635; opening cash 1 Jan 2027 lower by 364,753 because the bond line is collected and the premium paid in Oct-Nov 2026 rather than after the year end; January timing +376,823. Net cash from January -7,129. Bonding program tab of each plan workbook updated (row 19).</t>
+    <t xml:space="preserve">28 Oct 2026 (Chris): (1) Acama on its $22,072,845 GMP (Projects!B10; was $21,263,405) with actual bond figures: bond issued 12 Oct 2026, bond line $326,200 (invoice LV-2026-ACA-01), CBI premium $155,409 (invoice #024003), Krueger cash $561,958 (615 Holdings schedule 28 Oct); bond month Oct 2026 (was Dec 2026). (2) Staffing engine superintendent slots 6-10 priced at $160,000 (were at the assistant superintendent rate, $125,000); affects the Oct 2027 superintendent. FY2026 NI -14,345; FY2027 LV NI +14,638 (GMP fee +27,001 less superintendent -12,364); Krueger January payout 1,228,421 -&gt; 1,254,835; tax distribution 245,851 -&gt; 238,636; opening cash 1 Jan 2027 -364,753 (bond net cost now runs through cash in Oct-Nov 2026 instead of January).</t>
   </si>
   <si>
     <t xml:space="preserve">Check: consolidated NI less the model check (0 = ties)</t>
   </si>
   <si>
     <t xml:space="preserve">Check: LV NI less the model check (0 = ties)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check: Dec 2027 closing cash less Base Case Model row 383 Dec-27, less the $115 APA difference (0 = ties)</t>
   </si>
 </sst>
 </file>
@@ -1867,35 +1870,35 @@
       </c>
       <c r="G6" s="9" t="n">
         <f aca="false">LV!G6+LV!G7</f>
-        <v>1187324.25562138</v>
+        <v>1191181.62553618</v>
       </c>
       <c r="H6" s="9" t="n">
         <f aca="false">LV!H6+LV!H7</f>
-        <v>1281039.24562138</v>
+        <v>1284896.61553618</v>
       </c>
       <c r="I6" s="9" t="n">
         <f aca="false">LV!I6+LV!I7</f>
-        <v>1171298.79562138</v>
+        <v>1175156.16553618</v>
       </c>
       <c r="J6" s="9" t="n">
         <f aca="false">LV!J6+LV!J7</f>
-        <v>1308387.61772613</v>
+        <v>1312244.98764093</v>
       </c>
       <c r="K6" s="9" t="n">
         <f aca="false">LV!K6+LV!K7</f>
-        <v>1312692.91488505</v>
+        <v>1316550.28479984</v>
       </c>
       <c r="L6" s="9" t="n">
         <f aca="false">LV!L6+LV!L7</f>
-        <v>1460388.59488505</v>
+        <v>1464245.96479984</v>
       </c>
       <c r="M6" s="9" t="n">
         <f aca="false">LV!M6+LV!M7</f>
-        <v>1276861.67488505</v>
+        <v>1280719.04479985</v>
       </c>
       <c r="N6" s="10" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>13019185.4276136</v>
+        <v>13046187.0170172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1928,7 +1931,7 @@
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">LV!H26+LV!H46+LV!H49+LV!H50</f>
-        <v>-61690.6100000013</v>
+        <v>-61690.6099999994</v>
       </c>
       <c r="I7" s="9" t="n">
         <f aca="false">LV!I26+LV!I46+LV!I49+LV!I50</f>
@@ -1952,7 +1955,7 @@
       </c>
       <c r="N7" s="10" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>-514774.949999999</v>
+        <v>-514774.949999997</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2152,35 +2155,35 @@
       </c>
       <c r="G11" s="12" t="n">
         <f aca="false">SUM(G6:G10)</f>
-        <v>592271.695585263</v>
+        <v>596129.065500062</v>
       </c>
       <c r="H11" s="12" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>1235164.42509507</v>
+        <v>1239021.79500987</v>
       </c>
       <c r="I11" s="12" t="n">
         <f aca="false">SUM(I6:I10)</f>
-        <v>1131462.36509507</v>
+        <v>1135319.73500987</v>
       </c>
       <c r="J11" s="12" t="n">
         <f aca="false">SUM(J6:J10)</f>
-        <v>1050934.74381312</v>
+        <v>1054792.11372791</v>
       </c>
       <c r="K11" s="12" t="n">
         <f aca="false">SUM(K6:K10)</f>
-        <v>1082647.14849666</v>
+        <v>1086504.51841146</v>
       </c>
       <c r="L11" s="12" t="n">
         <f aca="false">SUM(L6:L10)</f>
-        <v>1476204.38435873</v>
+        <v>1480061.75427353</v>
       </c>
       <c r="M11" s="12" t="n">
         <f aca="false">SUM(M6:M10)</f>
-        <v>1350052.46435873</v>
+        <v>1353909.83427353</v>
       </c>
       <c r="N11" s="12" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>11277175.9774329</v>
+        <v>11304177.5668365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2758,35 +2761,35 @@
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">LV!G86</f>
-        <v>10578.0681115788</v>
+        <v>14435.4380263787</v>
       </c>
       <c r="H23" s="9" t="n">
         <f aca="false">LV!H86</f>
-        <v>720502.04762138</v>
+        <v>724359.417536182</v>
       </c>
       <c r="I23" s="9" t="n">
         <f aca="false">LV!I86</f>
-        <v>616799.987621384</v>
+        <v>620657.35753618</v>
       </c>
       <c r="J23" s="9" t="n">
         <f aca="false">LV!J86</f>
-        <v>536272.366339431</v>
+        <v>540129.736254229</v>
       </c>
       <c r="K23" s="9" t="n">
         <f aca="false">LV!K86</f>
-        <v>468173.521022977</v>
+        <v>472030.890937775</v>
       </c>
       <c r="L23" s="9" t="n">
         <f aca="false">LV!L86</f>
-        <v>843789.930435049</v>
+        <v>847647.300349847</v>
       </c>
       <c r="M23" s="9" t="n">
         <f aca="false">LV!M86</f>
-        <v>522828.836885048</v>
+        <v>526686.206799846</v>
       </c>
       <c r="N23" s="10" t="n">
         <f aca="false">SUM(B23:M23)</f>
-        <v>4725653.26603555</v>
+        <v>4752654.85543914</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2929,35 +2932,35 @@
       </c>
       <c r="G26" s="12" t="n">
         <f aca="false">SUM(G23:G25)</f>
-        <v>-145823.887414737</v>
+        <v>-141966.517499937</v>
       </c>
       <c r="H26" s="12" t="n">
         <f aca="false">SUM(H23:H25)</f>
-        <v>540193.842095064</v>
+        <v>544051.212009866</v>
       </c>
       <c r="I26" s="12" t="n">
         <f aca="false">SUM(I23:I25)</f>
-        <v>436491.782095068</v>
+        <v>440349.152009864</v>
       </c>
       <c r="J26" s="12" t="n">
         <f aca="false">SUM(J23:J25)</f>
-        <v>355964.160813115</v>
+        <v>359821.530727914</v>
       </c>
       <c r="K26" s="12" t="n">
         <f aca="false">SUM(K23:K25)</f>
-        <v>287865.315496661</v>
+        <v>291722.685411459</v>
       </c>
       <c r="L26" s="12" t="n">
         <f aca="false">SUM(L23:L25)</f>
-        <v>663481.724908734</v>
+        <v>667339.094823532</v>
       </c>
       <c r="M26" s="12" t="n">
         <f aca="false">SUM(M23:M25)</f>
-        <v>399895.631358732</v>
+        <v>403753.00127353</v>
       </c>
       <c r="N26" s="12" t="n">
         <f aca="false">SUM(B26:M26)</f>
-        <v>2751659.40498292</v>
+        <v>2778660.99438651</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3023,27 +3026,27 @@
       </c>
       <c r="H29" s="10" t="n">
         <f aca="false">G38</f>
-        <v>115418.095192296</v>
+        <v>115225.226696559</v>
       </c>
       <c r="I29" s="10" t="n">
         <f aca="false">H38</f>
-        <v>-74730.1145035123</v>
+        <v>-71258.4815801905</v>
       </c>
       <c r="J29" s="10" t="n">
         <f aca="false">I38</f>
-        <v>376361.715810486</v>
+        <v>383497.850152866</v>
       </c>
       <c r="K29" s="10" t="n">
         <f aca="false">J38</f>
-        <v>773392.719019244</v>
+        <v>784193.354780683</v>
       </c>
       <c r="L29" s="10" t="n">
         <f aca="false">K38</f>
-        <v>945058.751088111</v>
+        <v>959523.888268608</v>
       </c>
       <c r="M29" s="10" t="n">
         <f aca="false">L38</f>
-        <v>1030605.70039052</v>
+        <v>1048735.33899008</v>
       </c>
       <c r="N29" s="10" t="n">
         <f aca="false">B29</f>
@@ -3076,35 +3079,35 @@
       </c>
       <c r="G30" s="9" t="n">
         <f aca="false">G26</f>
-        <v>-145823.887414737</v>
+        <v>-141966.517499937</v>
       </c>
       <c r="H30" s="9" t="n">
         <f aca="false">H26</f>
-        <v>540193.842095064</v>
+        <v>544051.212009866</v>
       </c>
       <c r="I30" s="9" t="n">
         <f aca="false">I26</f>
-        <v>436491.782095068</v>
+        <v>440349.152009864</v>
       </c>
       <c r="J30" s="9" t="n">
         <f aca="false">J26</f>
-        <v>355964.160813115</v>
+        <v>359821.530727914</v>
       </c>
       <c r="K30" s="9" t="n">
         <f aca="false">K26</f>
-        <v>287865.315496661</v>
+        <v>291722.685411459</v>
       </c>
       <c r="L30" s="9" t="n">
         <f aca="false">L26</f>
-        <v>663481.724908734</v>
+        <v>667339.094823532</v>
       </c>
       <c r="M30" s="9" t="n">
         <f aca="false">M26</f>
-        <v>399895.631358732</v>
+        <v>403753.00127353</v>
       </c>
       <c r="N30" s="10" t="n">
         <f aca="false">SUM(B30:M30)</f>
-        <v>2751659.40498292</v>
+        <v>2778660.99438651</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3127,13 +3130,13 @@
         <v>-183650.08816422</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>97706.5504109574</v>
+        <v>93849.1804961603</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>-666290.089509803</v>
+        <v>-666290.089509806</v>
       </c>
       <c r="I31" s="9" t="n">
-        <v>104349.459999999</v>
+        <v>104349.460000001</v>
       </c>
       <c r="J31" s="9" t="n">
         <v>81033.4312819499</v>
@@ -3149,7 +3152,7 @@
       </c>
       <c r="N31" s="10" t="n">
         <f aca="false">SUM(B31:M31)</f>
-        <v>-737074.434885046</v>
+        <v>-740931.804799845</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3172,29 +3175,29 @@
         <v>-45256.9666161515</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>-59366.2127810691</v>
+        <v>-59559.081276809</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>-64051.9622810691</v>
+        <v>-64244.830776809</v>
       </c>
       <c r="I32" s="9" t="n">
-        <v>-58564.9397810691</v>
+        <v>-58757.808276809</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>-65419.3808863066</v>
+        <v>-65612.2493820466</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>-65634.6457442524</v>
+        <v>-65827.5142399922</v>
       </c>
       <c r="L32" s="9" t="n">
-        <v>-73019.4297442523</v>
+        <v>-73212.2982399922</v>
       </c>
       <c r="M32" s="9" t="n">
-        <v>-63843.0837442523</v>
+        <v>-64035.9522399922</v>
       </c>
       <c r="N32" s="10" t="n">
         <f aca="false">SUM(B32:M32)</f>
-        <v>-650959.271380679</v>
+        <v>-652309.350850858</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3403,35 +3406,35 @@
       </c>
       <c r="G37" s="10" t="n">
         <f aca="false">SUM(G30:G36)</f>
-        <v>-77056.0662848487</v>
+        <v>-77248.9347805858</v>
       </c>
       <c r="H37" s="10" t="n">
         <f aca="false">SUM(H30:H36)</f>
-        <v>-190148.209695808</v>
+        <v>-186483.708276749</v>
       </c>
       <c r="I37" s="10" t="n">
         <f aca="false">SUM(I30:I36)</f>
-        <v>451091.830313998</v>
+        <v>454756.331733056</v>
       </c>
       <c r="J37" s="10" t="n">
         <f aca="false">SUM(J30:J36)</f>
-        <v>397031.003208759</v>
+        <v>400695.504627817</v>
       </c>
       <c r="K37" s="10" t="n">
         <f aca="false">SUM(K30:K36)</f>
-        <v>171666.032068867</v>
+        <v>175330.533487925</v>
       </c>
       <c r="L37" s="10" t="n">
         <f aca="false">SUM(L30:L36)</f>
-        <v>85546.9493024112</v>
+        <v>89211.4507214694</v>
       </c>
       <c r="M37" s="10" t="n">
         <f aca="false">SUM(M30:M36)</f>
-        <v>408618.927614477</v>
+        <v>412283.429033535</v>
       </c>
       <c r="N37" s="10" t="n">
         <f aca="false">SUM(B37:M37)</f>
-        <v>-348911.910020011</v>
+        <v>-327117.770001398</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3460,35 +3463,35 @@
       </c>
       <c r="G38" s="12" t="n">
         <f aca="false">G29+G37</f>
-        <v>115418.095192296</v>
+        <v>115225.226696559</v>
       </c>
       <c r="H38" s="12" t="n">
         <f aca="false">H29+H37</f>
-        <v>-74730.1145035123</v>
+        <v>-71258.4815801905</v>
       </c>
       <c r="I38" s="12" t="n">
         <f aca="false">I29+I37</f>
-        <v>376361.715810486</v>
+        <v>383497.850152866</v>
       </c>
       <c r="J38" s="12" t="n">
         <f aca="false">J29+J37</f>
-        <v>773392.719019244</v>
+        <v>784193.354780683</v>
       </c>
       <c r="K38" s="12" t="n">
         <f aca="false">K29+K37</f>
-        <v>945058.751088111</v>
+        <v>959523.888268608</v>
       </c>
       <c r="L38" s="12" t="n">
         <f aca="false">L29+L37</f>
-        <v>1030605.70039052</v>
+        <v>1048735.33899008</v>
       </c>
       <c r="M38" s="12" t="n">
         <f aca="false">M29+M37</f>
-        <v>1439224.628005</v>
+        <v>1461018.76802361</v>
       </c>
       <c r="N38" s="12" t="n">
         <f aca="false">M38</f>
-        <v>1439224.628005</v>
+        <v>1461018.76802361</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,35 +3588,35 @@
       </c>
       <c r="G43" s="9" t="n">
         <f aca="false">LV!G27</f>
-        <v>8768040.94323706</v>
+        <v>8784632.04414071</v>
       </c>
       <c r="H43" s="9" t="n">
         <f aca="false">LV!H27</f>
-        <v>10144347.3730913</v>
+        <v>10164045.9158825</v>
       </c>
       <c r="I43" s="9" t="n">
         <f aca="false">LV!I27</f>
-        <v>9796181.31484267</v>
+        <v>9819205.84844292</v>
       </c>
       <c r="J43" s="9" t="n">
         <f aca="false">LV!J27</f>
-        <v>11103411.537929</v>
+        <v>11129908.5710597</v>
       </c>
       <c r="K43" s="9" t="n">
         <f aca="false">LV!K27</f>
-        <v>10990981.1829161</v>
+        <v>11021000.9008853</v>
       </c>
       <c r="L43" s="9" t="n">
         <f aca="false">LV!L27</f>
-        <v>12901723.7996864</v>
+        <v>12935208.732222</v>
       </c>
       <c r="M43" s="9" t="n">
         <f aca="false">LV!M27</f>
-        <v>11944082.569663</v>
+        <v>11980853.8304256</v>
       </c>
       <c r="N43" s="10" t="n">
         <f aca="false">SUM(B43:M43)</f>
-        <v>107112238.465346</v>
+        <v>107298325.58704</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3695,7 +3698,7 @@
       <c r="D6" s="20"/>
       <c r="E6" s="21" t="n">
         <f aca="false">Consolidated!N23</f>
-        <v>4725653.26603555</v>
+        <v>4752654.85543914</v>
       </c>
       <c r="F6" s="20"/>
     </row>
@@ -3734,7 +3737,7 @@
       <c r="D9" s="20"/>
       <c r="E9" s="24" t="n">
         <f aca="false">Consolidated!N26</f>
-        <v>2751659.40498292</v>
+        <v>2778660.99438651</v>
       </c>
       <c r="F9" s="20"/>
     </row>
@@ -3744,7 +3747,7 @@
       </c>
       <c r="E10" s="25" t="n">
         <f aca="false">MIN(Consolidated!B38:M38)</f>
-        <v>-74730.1145035123</v>
+        <v>-71258.4815801905</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>57</v>
@@ -3756,7 +3759,7 @@
       </c>
       <c r="E11" s="25" t="n">
         <f aca="false">Consolidated!M38</f>
-        <v>1439224.628005</v>
+        <v>1461018.76802361</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3959,7 +3962,7 @@
       </c>
       <c r="E26" s="9" t="n">
         <f aca="false">LV!N16</f>
-        <v>4179059.87119206</v>
+        <v>4338145.40348167</v>
       </c>
       <c r="F26" s="20"/>
     </row>
@@ -4140,7 +4143,7 @@
       </c>
       <c r="E36" s="31" t="n">
         <f aca="false">SUM(E19:E35)</f>
-        <v>94093053.0377328</v>
+        <v>94252138.5700224</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5193,29 +5196,29 @@
         <v>515376.770734153</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>677840.357636663</v>
+        <v>680044.573593741</v>
       </c>
       <c r="H6" s="39" t="n">
-        <v>731225.897636663</v>
+        <v>733430.113593741</v>
       </c>
       <c r="I6" s="39" t="n">
-        <v>668362.717636663</v>
+        <v>670566.933593741</v>
       </c>
       <c r="J6" s="39" t="n">
-        <v>742122.197550413</v>
+        <v>744326.413507491</v>
       </c>
       <c r="K6" s="39" t="n">
-        <v>745054.658202019</v>
+        <v>747258.874159097</v>
       </c>
       <c r="L6" s="39" t="n">
-        <v>826867.188202019</v>
+        <v>829071.404159097</v>
       </c>
       <c r="M6" s="39" t="n">
-        <v>724495.748202019</v>
+        <v>726699.964159097</v>
       </c>
       <c r="N6" s="40" t="n">
         <f aca="false">SUM(B6:M6)</f>
-        <v>7402425.19724927</v>
+        <v>7417854.70894881</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5238,29 +5241,29 @@
         <v>389762.561588878</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>509483.897984719</v>
+        <v>511137.05194244</v>
       </c>
       <c r="H7" s="39" t="n">
-        <v>549813.347984719</v>
+        <v>551466.50194244</v>
       </c>
       <c r="I7" s="39" t="n">
-        <v>502936.07798472</v>
+        <v>504589.23194244</v>
       </c>
       <c r="J7" s="39" t="n">
-        <v>566265.42017572</v>
+        <v>567918.57413344</v>
       </c>
       <c r="K7" s="39" t="n">
-        <v>567638.256683027</v>
+        <v>569291.410640747</v>
       </c>
       <c r="L7" s="39" t="n">
-        <v>633521.406683027</v>
+        <v>635174.560640747</v>
       </c>
       <c r="M7" s="39" t="n">
-        <v>552365.926683028</v>
+        <v>554019.080640748</v>
       </c>
       <c r="N7" s="40" t="n">
         <f aca="false">SUM(B7:M7)</f>
-        <v>5616760.23036432</v>
+        <v>5628332.30806836</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5616,29 +5619,29 @@
         <v>0</v>
       </c>
       <c r="G16" s="39" t="n">
-        <v>334505.743043865</v>
+        <v>347239.474032717</v>
       </c>
       <c r="H16" s="39" t="n">
-        <v>416135.954838865</v>
+        <v>431977.127715267</v>
       </c>
       <c r="I16" s="39" t="n">
-        <v>503507.285983865</v>
+        <v>522674.449669317</v>
       </c>
       <c r="J16" s="39" t="n">
-        <v>594727.293433865</v>
+        <v>617366.956649817</v>
       </c>
       <c r="K16" s="39" t="n">
-        <v>687265.631993865</v>
+        <v>713427.980048217</v>
       </c>
       <c r="L16" s="39" t="n">
-        <v>778294.268798865</v>
+        <v>807921.831419667</v>
       </c>
       <c r="M16" s="39" t="n">
-        <v>864623.693098865</v>
+        <v>897537.583946667</v>
       </c>
       <c r="N16" s="40" t="n">
         <f aca="false">SUM(B16:M16)</f>
-        <v>4179059.87119206</v>
+        <v>4338145.40348167</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6072,35 +6075,35 @@
       </c>
       <c r="G26" s="40" t="n">
         <f aca="false">G9+G10+G11+G12+G13+G14+G15+G16+G17+G18+G19+G20+G21+G22+G23+G24+G25</f>
-        <v>7580716.68761567</v>
+        <v>7593450.41860453</v>
       </c>
       <c r="H26" s="40" t="n">
         <f aca="false">H9+H10+H11+H12+H13+H14+H15+H16+H17+H18+H19+H20+H21+H22+H23+H24+H25</f>
-        <v>8863308.12746995</v>
+        <v>8879149.30034635</v>
       </c>
       <c r="I26" s="40" t="n">
         <f aca="false">I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24+I25</f>
-        <v>8624882.51922129</v>
+        <v>8644049.68290674</v>
       </c>
       <c r="J26" s="40" t="n">
         <f aca="false">J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25</f>
-        <v>9795023.92020283</v>
+        <v>9817663.58341878</v>
       </c>
       <c r="K26" s="40" t="n">
         <f aca="false">K9+K10+K11+K12+K13+K14+K15+K16+K17+K18+K19+K20+K21+K22+K23+K24+K25</f>
-        <v>9678288.26803106</v>
+        <v>9704450.61608541</v>
       </c>
       <c r="L26" s="40" t="n">
         <f aca="false">L9+L10+L11+L12+L13+L14+L15+L16+L17+L18+L19+L20+L21+L22+L23+L24+L25</f>
-        <v>11441335.2048013</v>
+        <v>11470962.7674221</v>
       </c>
       <c r="M26" s="40" t="n">
         <f aca="false">M9+M10+M11+M12+M13+M14+M15+M16+M17+M18+M19+M20+M21+M22+M23+M24+M25</f>
-        <v>10667220.8947779</v>
+        <v>10700134.7856257</v>
       </c>
       <c r="N26" s="40" t="n">
         <f aca="false">N9+N10+N11+N12+N13+N14+N15+N16+N17+N18+N19+N20+N21+N22+N23+N24+N25</f>
-        <v>94093053.0377328</v>
+        <v>94252138.5700224</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6129,35 +6132,35 @@
       </c>
       <c r="G27" s="43" t="n">
         <f aca="false">G6+G7+G26</f>
-        <v>8768040.94323706</v>
+        <v>8784632.04414071</v>
       </c>
       <c r="H27" s="43" t="n">
         <f aca="false">H6+H7+H26</f>
-        <v>10144347.3730913</v>
+        <v>10164045.9158825</v>
       </c>
       <c r="I27" s="43" t="n">
         <f aca="false">I6+I7+I26</f>
-        <v>9796181.31484267</v>
+        <v>9819205.84844292</v>
       </c>
       <c r="J27" s="43" t="n">
         <f aca="false">J6+J7+J26</f>
-        <v>11103411.537929</v>
+        <v>11129908.5710597</v>
       </c>
       <c r="K27" s="43" t="n">
         <f aca="false">K6+K7+K26</f>
-        <v>10990981.1829161</v>
+        <v>11021000.9008853</v>
       </c>
       <c r="L27" s="43" t="n">
         <f aca="false">L6+L7+L26</f>
-        <v>12901723.7996864</v>
+        <v>12935208.732222</v>
       </c>
       <c r="M27" s="43" t="n">
         <f aca="false">M6+M7+M26</f>
-        <v>11944082.569663</v>
+        <v>11980853.8304256</v>
       </c>
       <c r="N27" s="43" t="n">
         <f aca="false">N6+N7+N26</f>
-        <v>107112238.465346</v>
+        <v>107298325.58704</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6513,29 +6516,29 @@
         <v>0</v>
       </c>
       <c r="G36" s="39" t="n">
-        <v>-334505.743043865</v>
+        <v>-347239.474032717</v>
       </c>
       <c r="H36" s="39" t="n">
-        <v>-416135.954838865</v>
+        <v>-431977.127715267</v>
       </c>
       <c r="I36" s="39" t="n">
-        <v>-503507.285983865</v>
+        <v>-522674.449669317</v>
       </c>
       <c r="J36" s="39" t="n">
-        <v>-594727.293433865</v>
+        <v>-617366.956649817</v>
       </c>
       <c r="K36" s="39" t="n">
-        <v>-687265.631993865</v>
+        <v>-713427.980048217</v>
       </c>
       <c r="L36" s="39" t="n">
-        <v>-778294.268798865</v>
+        <v>-807921.831419667</v>
       </c>
       <c r="M36" s="39" t="n">
-        <v>-864623.693098865</v>
+        <v>-897537.583946667</v>
       </c>
       <c r="N36" s="40" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>-4179059.87119206</v>
+        <v>-4338145.40348167</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6969,35 +6972,35 @@
       </c>
       <c r="G46" s="40" t="n">
         <f aca="false">G29+G30+G31+G32+G33+G34+G35+G36+G37+G38+G39+G40+G41+G42+G43+G44+G45</f>
-        <v>-7631396.09761567</v>
+        <v>-7644129.82860453</v>
       </c>
       <c r="H46" s="40" t="n">
         <f aca="false">H29+H30+H31+H32+H33+H34+H35+H36+H37+H38+H39+H40+H41+H42+H43+H44+H45</f>
-        <v>-8924351.33746995</v>
+        <v>-8940192.51034635</v>
       </c>
       <c r="I46" s="40" t="n">
         <f aca="false">I29+I30+I31+I32+I33+I34+I35+I36+I37+I38+I39+I40+I41+I42+I43+I44+I45</f>
-        <v>-8680028.92922129</v>
+        <v>-8699196.09290674</v>
       </c>
       <c r="J46" s="40" t="n">
         <f aca="false">J29+J30+J31+J32+J33+J34+J35+J36+J37+J38+J39+J40+J41+J42+J43+J44+J45</f>
-        <v>-9815388.53020283</v>
+        <v>-9838028.19341878</v>
       </c>
       <c r="K46" s="40" t="n">
         <f aca="false">K29+K30+K31+K32+K33+K34+K35+K36+K37+K38+K39+K40+K41+K42+K43+K44+K45</f>
-        <v>-9680614.65803106</v>
+        <v>-9706777.00608541</v>
       </c>
       <c r="L46" s="40" t="n">
         <f aca="false">L29+L30+L31+L32+L33+L34+L35+L36+L37+L38+L39+L40+L41+L42+L43+L44+L45</f>
-        <v>-11440295.7448013</v>
+        <v>-11469923.3074221</v>
       </c>
       <c r="M46" s="40" t="n">
         <f aca="false">M29+M30+M31+M32+M33+M34+M35+M36+M37+M38+M39+M40+M41+M42+M43+M44+M45</f>
-        <v>-10666570.7147779</v>
+        <v>-10699484.6056257</v>
       </c>
       <c r="N46" s="40" t="n">
         <f aca="false">N29+N30+N31+N32+N33+N34+N35+N36+N37+N38+N39+N40+N41+N42+N43+N44+N45</f>
-        <v>-94600524.8677328</v>
+        <v>-94759610.4000224</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7179,35 +7182,35 @@
       </c>
       <c r="G51" s="43" t="n">
         <f aca="false">G27+G46+G48+G49+G50</f>
-        <v>552549.656111579</v>
+        <v>556407.026026379</v>
       </c>
       <c r="H51" s="43" t="n">
         <f aca="false">H27+H46+H48+H49+H50</f>
-        <v>1219348.63562138</v>
+        <v>1223206.00553618</v>
       </c>
       <c r="I51" s="43" t="n">
         <f aca="false">I27+I46+I48+I49+I50</f>
-        <v>1115646.57562138</v>
+        <v>1119503.94553618</v>
       </c>
       <c r="J51" s="43" t="n">
         <f aca="false">J27+J46+J48+J49+J50</f>
-        <v>1035118.95433943</v>
+        <v>1038976.32425423</v>
       </c>
       <c r="K51" s="43" t="n">
         <f aca="false">K27+K46+K48+K49+K50</f>
-        <v>1066831.35902298</v>
+        <v>1070688.72893778</v>
       </c>
       <c r="L51" s="43" t="n">
         <f aca="false">L27+L46+L48+L49+L50</f>
-        <v>1460388.59488505</v>
+        <v>1464245.96479985</v>
       </c>
       <c r="M51" s="43" t="n">
         <f aca="false">M27+M46+M48+M49+M50</f>
-        <v>1276861.67488505</v>
+        <v>1280719.04479985</v>
       </c>
       <c r="N51" s="43" t="n">
         <f aca="false">N27+N46+N48+N49+N50</f>
-        <v>10888931.8984856</v>
+        <v>10915933.4878891</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8751,35 +8754,35 @@
       </c>
       <c r="G86" s="43" t="n">
         <f aca="false">G51+G85</f>
-        <v>10578.0681115788</v>
+        <v>14435.4380263787</v>
       </c>
       <c r="H86" s="43" t="n">
         <f aca="false">H51+H85</f>
-        <v>720502.04762138</v>
+        <v>724359.417536182</v>
       </c>
       <c r="I86" s="43" t="n">
         <f aca="false">I51+I85</f>
-        <v>616799.987621384</v>
+        <v>620657.35753618</v>
       </c>
       <c r="J86" s="43" t="n">
         <f aca="false">J51+J85</f>
-        <v>536272.366339431</v>
+        <v>540129.736254229</v>
       </c>
       <c r="K86" s="43" t="n">
         <f aca="false">K51+K85</f>
-        <v>468173.521022977</v>
+        <v>472030.890937775</v>
       </c>
       <c r="L86" s="43" t="n">
         <f aca="false">L51+L85</f>
-        <v>843789.930435049</v>
+        <v>847647.300349847</v>
       </c>
       <c r="M86" s="43" t="n">
         <f aca="false">M51+M85</f>
-        <v>522828.836885048</v>
+        <v>526686.206799846</v>
       </c>
       <c r="N86" s="43" t="n">
         <f aca="false">N51+N85</f>
-        <v>4725653.26603555</v>
+        <v>4752654.85543912</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -11584,7 +11587,7 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">Consolidated!N23</f>
-        <v>4725653.26603555</v>
+        <v>4752654.85543914</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">-D11</f>
@@ -11592,7 +11595,7 @@
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">B15+C15</f>
-        <v>3790783.51603555</v>
+        <v>3817785.10543914</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11634,7 +11637,7 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">SUM(B15:B17)</f>
-        <v>2751659.40498292</v>
+        <v>2778660.99438651</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">SUM(C15:C17)</f>
@@ -11642,7 +11645,7 @@
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">SUM(D15:D17)</f>
-        <v>2751659.40498292</v>
+        <v>2778660.99438651</v>
       </c>
     </row>
   </sheetData>
@@ -11665,7 +11668,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="60"/>
@@ -11703,7 +11706,7 @@
         <v>334</v>
       </c>
       <c r="B5" s="49" t="n">
-        <v>4725653</v>
+        <v>4752655</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11733,7 +11736,7 @@
         <v>338</v>
       </c>
       <c r="B9" s="49" t="n">
-        <v>2751660</v>
+        <v>2778661</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11849,7 +11852,7 @@
       </c>
       <c r="B30" s="1" t="n">
         <f aca="false">ROUND(Consolidated!N26-B9,0)</f>
-        <v>-1</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11858,7 +11861,16 @@
       </c>
       <c r="B31" s="1" t="n">
         <f aca="false">ROUND(Consolidated!N23-B5,0)</f>
-        <v>0</v>
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="B32" s="1" t="n">
+        <f aca="false">ROUND(Consolidated!M38-(1461134-115),0)</f>
+        <v>-0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Board portal: Andresen FY2026 bridge, 12th & Fir at $8,800/mo, staffing vs active jobs; fix GMP 'was' note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EkVDtrr64Hp1gx17meyeHf
</commit_message>
<xml_diff>
--- a/models/SixPeak_OperatingBudget_2026-10-28.xlsx
+++ b/models/SixPeak_OperatingBudget_2026-10-28.xlsx
@@ -11,10 +11,11 @@
     <sheet name="Consolidated" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Key Assumptions" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="LV" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Six Peak" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="APA" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Mgmt View (Hypothetical)" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Source and checks" sheetId="7" state="hidden" r:id="rId9"/>
+    <sheet name="Staffing" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Six Peak" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="APA" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Mgmt View (Hypothetical)" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Source and checks" sheetId="8" state="hidden" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="424">
   <si>
     <t xml:space="preserve">Six Peak consolidated FY2027 budget</t>
   </si>
@@ -826,6 +827,195 @@
     <t xml:space="preserve">LV NET INCOME</t>
   </si>
   <si>
+    <t xml:space="preserve">LV staffing: active jobs and people by role, April 2026 to December 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requested by Chris Andresen (29 Oct 2026) to explain the FY2027 hires, the main expense item. Source: Base Case staffing engine and Personnel tab (models _2026-10-28). April 2026 is the first month of the model roster; payroll staffing schedules before June list only part of the team, so earlier months are not shown. "Needed" is the engine's requirement from the active jobs, including superintendent lead time before a start; a role is hired only when the need exceeds staff by 0.75 of a person, and PMs and APMs overlap a job's last 5 months.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apr 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dec 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jan 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feb 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mar 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apr 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jul 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oct 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nov 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dec 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active jobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People on staff, by role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Project managers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      needed for the active jobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Assistant project managers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Superintendents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Assistant superintendents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Project coordinators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Operations and labor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Executives and office</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total people on staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Change in headcount (hires less departures)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LV payroll, 5000-1000 (incl. December bonus pool)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payroll per active job</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active jobs per project manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 versus 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 (Apr to Dec)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average active jobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active jobs at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average people on staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People on staff at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Project managers, year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Assistant project managers, year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Superintendents, year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Assistant superintendents, year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Project coordinators, year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Operations and labor, year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Executives and office, year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average active jobs per project manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average active jobs per superintendent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LV payroll per active job, per month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading it: active jobs roughly double (about 6.6 a month on average from April to December 2026, about 12 in 2027) while people on staff grow by about 40%. Hiring follows job starts; it is not running ahead of them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payroll per active job falls from about $38K a month to about $30K: the team is stretched further in 2027, mostly on project managers (about 2.2 jobs each in 2026, 3.7 in 2027).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superintendents stay at about one per job. The thin months are February to June 2027, when starts run ahead of hires; PMs and APMs cover.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Executives and office drops by one in January 2027: Joe LaKamp retires December 31.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hires are roles tied to job starts. If an award slips or is lost, its hires move or drop with it (Projects tab Active switch).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Six Peak Capital: draft FY2027 budget</t>
   </si>
   <si>
@@ -1099,7 +1289,7 @@
     <t xml:space="preserve">What-moves-it figures rerun 26 Oct 2026 on the final Base Case (models _2026-10-26): Reseda off -320,878; Beverly off -97,401; Acama at the Dec 2026 start +409,364 (so the slip costs 409,364).</t>
   </si>
   <si>
-    <t xml:space="preserve">28 Oct 2026 (Chris): (1) Acama on its $22,072,845 GMP (Projects!B10; was $21,263,405) with actual bond figures: bond issued 12 Oct 2026, bond line $326,200 (invoice LV-2026-ACA-01), CBI premium $155,409 (invoice #024003), Krueger cash $561,958 (615 Holdings schedule 28 Oct); bond month Oct 2026 (was Dec 2026). (2) Staffing engine superintendent slots 6-10 priced at $160,000 (were at the assistant superintendent rate, $125,000); affects the Oct 2027 superintendent. FY2026 NI -14,345; FY2027 LV NI +14,638 (GMP fee +27,001 less superintendent -12,364); Krueger January payout 1,228,421 -&gt; 1,254,835; tax distribution 245,851 -&gt; 238,636; opening cash 1 Jan 2027 -364,753 (bond net cost now runs through cash in Oct-Nov 2026 instead of January).</t>
+    <t xml:space="preserve">28 Oct 2026 (Chris): (1) Acama on its $22,072,845 GMP (Projects!B10; was $21,263,405) with actual bond figures: bond issued 12 Oct 2026, bond line $326,200 (invoice LV-2026-ACA-01), CBI premium $155,409 (invoice #024003), Krueger cash $561,958 (615 Holdings schedule 28 Oct); bond month Oct 2026 (was Dec 2026). (2) 12th &amp; Fir developer fee $8,800 a month (was $9,500), Jul 2026 to Sep 2028 (Chris Andresen, 29 Oct). (3) Staffing engine superintendent slots 6-10 priced at $160,000 (were at the assistant superintendent rate, $125,000); affects the Oct 2027 superintendent. FY2026 NI -14,345; FY2027 LV NI +14,638 (GMP fee +27,001 less superintendent -12,364); Krueger January payout 1,228,421 -&gt; 1,254,835; tax distribution 245,851 -&gt; 238,636; opening cash 1 Jan 2027 -364,753 (bond net cost now runs through cash in Oct-Nov 2026 instead of January).</t>
   </si>
   <si>
     <t xml:space="preserve">Check: consolidated NI less the model check (0 = ties)</t>
@@ -1115,14 +1305,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0.00,,\M;&quot;($&quot;#,##0.00,,&quot;M)&quot;"/>
     <numFmt numFmtId="167" formatCode="\$#,##0"/>
-    <numFmt numFmtId="168" formatCode="0%"/>
+    <numFmt numFmtId="168" formatCode="0.0;\(0.0\);\-"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="0.00"/>
+    <numFmt numFmtId="171" formatCode="0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Aptos"/>
@@ -1214,8 +1407,23 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF6B7280"/>
+      <name val="Aptos"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
+      <name val="Aptos"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF0B1833"/>
       <name val="Aptos"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1248,7 +1456,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1285,6 +1493,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF0B1833"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1311,7 +1528,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="69">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1488,7 +1705,83 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1496,7 +1789,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1504,7 +1797,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1569,12 +1862,12 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF475569"/>
+      <rgbColor rgb="FF6B7280"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF0B1833"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF475569"/>
       <rgbColor rgb="FFA84A15"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF1F4E9A"/>
@@ -2021,55 +2314,55 @@
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">'Six Peak'!B11</f>
-        <v>36564.1447368421</v>
+        <v>35864.1447368421</v>
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">'Six Peak'!C11</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">'Six Peak'!D11</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">'Six Peak'!E11</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="F9" s="9" t="n">
         <f aca="false">'Six Peak'!F11</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="G9" s="9" t="n">
         <f aca="false">'Six Peak'!G11</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="H9" s="9" t="n">
         <f aca="false">'Six Peak'!H11</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="I9" s="9" t="n">
         <f aca="false">'Six Peak'!I11</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="J9" s="9" t="n">
         <f aca="false">'Six Peak'!J11</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="K9" s="9" t="n">
         <f aca="false">'Six Peak'!K11</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="L9" s="9" t="n">
         <f aca="false">'Six Peak'!L11</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="M9" s="9" t="n">
         <f aca="false">'Six Peak'!M11</f>
-        <v>73190.7894736842</v>
+        <v>72490.7894736842</v>
       </c>
       <c r="N9" s="10" t="n">
         <f aca="false">SUM(B9:M9)</f>
-        <v>387444.078947369</v>
+        <v>379044.078947369</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2135,55 +2428,55 @@
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">SUM(B6:B10)</f>
-        <v>693183.051455493</v>
+        <v>692483.051455493</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">SUM(C6:C10)</f>
-        <v>725601.962673285</v>
+        <v>724901.962673285</v>
       </c>
       <c r="D11" s="12" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>744876.582673284</v>
+        <v>744176.582673284</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>505323.007832</v>
+        <v>504623.007832</v>
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">SUM(F6:F10)</f>
-        <v>689454.14599622</v>
+        <v>688754.14599622</v>
       </c>
       <c r="G11" s="12" t="n">
         <f aca="false">SUM(G6:G10)</f>
-        <v>596129.065500062</v>
+        <v>595429.065500062</v>
       </c>
       <c r="H11" s="12" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>1239021.79500987</v>
+        <v>1238321.79500987</v>
       </c>
       <c r="I11" s="12" t="n">
         <f aca="false">SUM(I6:I10)</f>
-        <v>1135319.73500987</v>
+        <v>1134619.73500987</v>
       </c>
       <c r="J11" s="12" t="n">
         <f aca="false">SUM(J6:J10)</f>
-        <v>1054792.11372791</v>
+        <v>1054092.11372791</v>
       </c>
       <c r="K11" s="12" t="n">
         <f aca="false">SUM(K6:K10)</f>
-        <v>1086504.51841146</v>
+        <v>1085804.51841146</v>
       </c>
       <c r="L11" s="12" t="n">
         <f aca="false">SUM(L6:L10)</f>
-        <v>1480061.75427353</v>
+        <v>1479361.75427353</v>
       </c>
       <c r="M11" s="12" t="n">
         <f aca="false">SUM(M6:M10)</f>
-        <v>1353909.83427353</v>
+        <v>1353209.83427353</v>
       </c>
       <c r="N11" s="12" t="n">
         <f aca="false">SUM(B11:M11)</f>
-        <v>11304177.5668365</v>
+        <v>11295777.5668365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2798,55 +3091,55 @@
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">'Six Peak'!B38</f>
-        <v>-163059.850263158</v>
+        <v>-163759.850263158</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">'Six Peak'!C38</f>
-        <v>-158151.955526316</v>
+        <v>-158851.955526316</v>
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">'Six Peak'!D38</f>
-        <v>-158151.955526316</v>
+        <v>-158851.955526316</v>
       </c>
       <c r="E24" s="9" t="n">
         <f aca="false">'Six Peak'!E38</f>
-        <v>-158151.955526316</v>
+        <v>-158851.955526316</v>
       </c>
       <c r="F24" s="9" t="n">
         <f aca="false">'Six Peak'!F38</f>
-        <v>-156401.955526316</v>
+        <v>-157101.955526316</v>
       </c>
       <c r="G24" s="9" t="n">
         <f aca="false">'Six Peak'!G38</f>
-        <v>-156401.955526316</v>
+        <v>-157101.955526316</v>
       </c>
       <c r="H24" s="9" t="n">
         <f aca="false">'Six Peak'!H38</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="I24" s="9" t="n">
         <f aca="false">'Six Peak'!I38</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="J24" s="9" t="n">
         <f aca="false">'Six Peak'!J38</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="K24" s="9" t="n">
         <f aca="false">'Six Peak'!K38</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="L24" s="9" t="n">
         <f aca="false">'Six Peak'!L38</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="M24" s="9" t="n">
         <f aca="false">'Six Peak'!M38</f>
-        <v>-122933.205526316</v>
+        <v>-123633.205526316</v>
       </c>
       <c r="N24" s="10" t="n">
         <f aca="false">SUM(B24:M24)</f>
-        <v>-1974793.86105263</v>
+        <v>-1983193.86105263</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2912,55 +3205,55 @@
       </c>
       <c r="B26" s="12" t="n">
         <f aca="false">SUM(B23:B25)</f>
-        <v>77411.2184554924</v>
+        <v>76711.2184554924</v>
       </c>
       <c r="C26" s="12" t="n">
         <f aca="false">SUM(C23:C25)</f>
-        <v>90611.3796732849</v>
+        <v>89911.3796732849</v>
       </c>
       <c r="D26" s="12" t="n">
         <f aca="false">SUM(D23:D25)</f>
-        <v>142760.999673283</v>
+        <v>142060.999673283</v>
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">SUM(E23:E25)</f>
-        <v>-123632.575168</v>
+        <v>-124332.575168</v>
       </c>
       <c r="F26" s="12" t="n">
         <f aca="false">SUM(F23:F25)</f>
-        <v>26439.8129962189</v>
+        <v>25739.8129962189</v>
       </c>
       <c r="G26" s="12" t="n">
         <f aca="false">SUM(G23:G25)</f>
-        <v>-141966.517499937</v>
+        <v>-142666.517499937</v>
       </c>
       <c r="H26" s="12" t="n">
         <f aca="false">SUM(H23:H25)</f>
-        <v>544051.212009866</v>
+        <v>543351.212009866</v>
       </c>
       <c r="I26" s="12" t="n">
         <f aca="false">SUM(I23:I25)</f>
-        <v>440349.152009864</v>
+        <v>439649.152009864</v>
       </c>
       <c r="J26" s="12" t="n">
         <f aca="false">SUM(J23:J25)</f>
-        <v>359821.530727914</v>
+        <v>359121.530727914</v>
       </c>
       <c r="K26" s="12" t="n">
         <f aca="false">SUM(K23:K25)</f>
-        <v>291722.685411459</v>
+        <v>291022.685411459</v>
       </c>
       <c r="L26" s="12" t="n">
         <f aca="false">SUM(L23:L25)</f>
-        <v>667339.094823532</v>
+        <v>666639.094823532</v>
       </c>
       <c r="M26" s="12" t="n">
         <f aca="false">SUM(M23:M25)</f>
-        <v>403753.00127353</v>
+        <v>403053.00127353</v>
       </c>
       <c r="N26" s="12" t="n">
         <f aca="false">SUM(B26:M26)</f>
-        <v>2778660.99438651</v>
+        <v>2770260.99438651</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3002,55 +3295,55 @@
         <v>38</v>
       </c>
       <c r="B29" s="10" t="n">
-        <v>1788136.53802501</v>
+        <v>1786036.53802501</v>
       </c>
       <c r="C29" s="10" t="n">
         <f aca="false">B38</f>
-        <v>212118.421188719</v>
+        <v>210374.721188719</v>
       </c>
       <c r="D29" s="10" t="n">
         <f aca="false">C38</f>
-        <v>236515.681721073</v>
+        <v>234071.981721074</v>
       </c>
       <c r="E29" s="10" t="n">
         <f aca="false">D38</f>
-        <v>322370.733734376</v>
+        <v>319227.033734377</v>
       </c>
       <c r="F29" s="10" t="n">
         <f aca="false">E38</f>
-        <v>394941.403261297</v>
+        <v>391097.703261298</v>
       </c>
       <c r="G29" s="10" t="n">
         <f aca="false">F38</f>
-        <v>192474.161477145</v>
+        <v>187930.461477145</v>
       </c>
       <c r="H29" s="10" t="n">
         <f aca="false">G38</f>
-        <v>115225.226696559</v>
+        <v>109981.526696559</v>
       </c>
       <c r="I29" s="10" t="n">
         <f aca="false">H38</f>
-        <v>-71258.4815801905</v>
+        <v>-77202.1815801902</v>
       </c>
       <c r="J29" s="10" t="n">
         <f aca="false">I38</f>
-        <v>383497.850152866</v>
+        <v>376854.150152866</v>
       </c>
       <c r="K29" s="10" t="n">
         <f aca="false">J38</f>
-        <v>784193.354780683</v>
+        <v>776849.654780683</v>
       </c>
       <c r="L29" s="10" t="n">
         <f aca="false">K38</f>
-        <v>959523.888268608</v>
+        <v>951480.188268608</v>
       </c>
       <c r="M29" s="10" t="n">
         <f aca="false">L38</f>
-        <v>1048735.33899008</v>
+        <v>1039991.63899008</v>
       </c>
       <c r="N29" s="10" t="n">
         <f aca="false">B29</f>
-        <v>1788136.53802501</v>
+        <v>1786036.53802501</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3059,55 +3352,55 @@
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">B26</f>
-        <v>77411.2184554924</v>
+        <v>76711.2184554924</v>
       </c>
       <c r="C30" s="9" t="n">
         <f aca="false">C26</f>
-        <v>90611.3796732849</v>
+        <v>89911.3796732849</v>
       </c>
       <c r="D30" s="9" t="n">
         <f aca="false">D26</f>
-        <v>142760.999673283</v>
+        <v>142060.999673283</v>
       </c>
       <c r="E30" s="9" t="n">
         <f aca="false">E26</f>
-        <v>-123632.575168</v>
+        <v>-124332.575168</v>
       </c>
       <c r="F30" s="9" t="n">
         <f aca="false">F26</f>
-        <v>26439.8129962189</v>
+        <v>25739.8129962189</v>
       </c>
       <c r="G30" s="9" t="n">
         <f aca="false">G26</f>
-        <v>-141966.517499937</v>
+        <v>-142666.517499937</v>
       </c>
       <c r="H30" s="9" t="n">
         <f aca="false">H26</f>
-        <v>544051.212009866</v>
+        <v>543351.212009866</v>
       </c>
       <c r="I30" s="9" t="n">
         <f aca="false">I26</f>
-        <v>440349.152009864</v>
+        <v>439649.152009864</v>
       </c>
       <c r="J30" s="9" t="n">
         <f aca="false">J26</f>
-        <v>359821.530727914</v>
+        <v>359121.530727914</v>
       </c>
       <c r="K30" s="9" t="n">
         <f aca="false">K26</f>
-        <v>291722.685411459</v>
+        <v>291022.685411459</v>
       </c>
       <c r="L30" s="9" t="n">
         <f aca="false">L26</f>
-        <v>667339.094823532</v>
+        <v>666639.094823532</v>
       </c>
       <c r="M30" s="9" t="n">
         <f aca="false">M26</f>
-        <v>403753.00127353</v>
+        <v>403053.00127353</v>
       </c>
       <c r="N30" s="10" t="n">
         <f aca="false">SUM(B30:M30)</f>
-        <v>2778660.99438651</v>
+        <v>2770260.99438651</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3340,7 +3633,7 @@
         <v>45</v>
       </c>
       <c r="B36" s="9" t="n">
-        <v>-238635.906987201</v>
+        <v>-237579.606987201</v>
       </c>
       <c r="C36" s="9" t="n">
         <v>0</v>
@@ -3377,7 +3670,7 @@
       </c>
       <c r="N36" s="10" t="n">
         <f aca="false">SUM(B36:M36)</f>
-        <v>-238635.906987201</v>
+        <v>-237579.606987201</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3386,55 +3679,55 @@
       </c>
       <c r="B37" s="10" t="n">
         <f aca="false">SUM(B30:B36)</f>
-        <v>-1576018.11683629</v>
+        <v>-1575661.81683629</v>
       </c>
       <c r="C37" s="10" t="n">
         <f aca="false">SUM(C30:C36)</f>
-        <v>24397.2605323548</v>
+        <v>23697.2605323548</v>
       </c>
       <c r="D37" s="10" t="n">
         <f aca="false">SUM(D30:D36)</f>
-        <v>85855.052013303</v>
+        <v>85155.052013303</v>
       </c>
       <c r="E37" s="10" t="n">
         <f aca="false">SUM(E30:E36)</f>
-        <v>72570.6695269209</v>
+        <v>71870.6695269209</v>
       </c>
       <c r="F37" s="10" t="n">
         <f aca="false">SUM(F30:F36)</f>
-        <v>-202467.241784153</v>
+        <v>-203167.241784153</v>
       </c>
       <c r="G37" s="10" t="n">
         <f aca="false">SUM(G30:G36)</f>
-        <v>-77248.9347805858</v>
+        <v>-77948.9347805858</v>
       </c>
       <c r="H37" s="10" t="n">
         <f aca="false">SUM(H30:H36)</f>
-        <v>-186483.708276749</v>
+        <v>-187183.708276749</v>
       </c>
       <c r="I37" s="10" t="n">
         <f aca="false">SUM(I30:I36)</f>
-        <v>454756.331733056</v>
+        <v>454056.331733056</v>
       </c>
       <c r="J37" s="10" t="n">
         <f aca="false">SUM(J30:J36)</f>
-        <v>400695.504627817</v>
+        <v>399995.504627817</v>
       </c>
       <c r="K37" s="10" t="n">
         <f aca="false">SUM(K30:K36)</f>
-        <v>175330.533487925</v>
+        <v>174630.533487925</v>
       </c>
       <c r="L37" s="10" t="n">
         <f aca="false">SUM(L30:L36)</f>
-        <v>89211.4507214694</v>
+        <v>88511.4507214694</v>
       </c>
       <c r="M37" s="10" t="n">
         <f aca="false">SUM(M30:M36)</f>
-        <v>412283.429033535</v>
+        <v>411583.429033535</v>
       </c>
       <c r="N37" s="10" t="n">
         <f aca="false">SUM(B37:M37)</f>
-        <v>-327117.770001398</v>
+        <v>-334461.470001398</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3443,55 +3736,55 @@
       </c>
       <c r="B38" s="12" t="n">
         <f aca="false">B29+B37</f>
-        <v>212118.421188719</v>
+        <v>210374.721188719</v>
       </c>
       <c r="C38" s="12" t="n">
         <f aca="false">C29+C37</f>
-        <v>236515.681721073</v>
+        <v>234071.981721074</v>
       </c>
       <c r="D38" s="12" t="n">
         <f aca="false">D29+D37</f>
-        <v>322370.733734376</v>
+        <v>319227.033734377</v>
       </c>
       <c r="E38" s="12" t="n">
         <f aca="false">E29+E37</f>
-        <v>394941.403261297</v>
+        <v>391097.703261298</v>
       </c>
       <c r="F38" s="12" t="n">
         <f aca="false">F29+F37</f>
-        <v>192474.161477145</v>
+        <v>187930.461477145</v>
       </c>
       <c r="G38" s="12" t="n">
         <f aca="false">G29+G37</f>
-        <v>115225.226696559</v>
+        <v>109981.526696559</v>
       </c>
       <c r="H38" s="12" t="n">
         <f aca="false">H29+H37</f>
-        <v>-71258.4815801905</v>
+        <v>-77202.1815801902</v>
       </c>
       <c r="I38" s="12" t="n">
         <f aca="false">I29+I37</f>
-        <v>383497.850152866</v>
+        <v>376854.150152866</v>
       </c>
       <c r="J38" s="12" t="n">
         <f aca="false">J29+J37</f>
-        <v>784193.354780683</v>
+        <v>776849.654780683</v>
       </c>
       <c r="K38" s="12" t="n">
         <f aca="false">K29+K37</f>
-        <v>959523.888268608</v>
+        <v>951480.188268608</v>
       </c>
       <c r="L38" s="12" t="n">
         <f aca="false">L29+L37</f>
-        <v>1048735.33899008</v>
+        <v>1039991.63899008</v>
       </c>
       <c r="M38" s="12" t="n">
         <f aca="false">M29+M37</f>
-        <v>1461018.76802361</v>
+        <v>1451575.06802361</v>
       </c>
       <c r="N38" s="12" t="n">
         <f aca="false">M38</f>
-        <v>1461018.76802361</v>
+        <v>1451575.06802361</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3711,7 +4004,7 @@
       <c r="D7" s="20"/>
       <c r="E7" s="21" t="n">
         <f aca="false">Consolidated!N24</f>
-        <v>-1974793.86105263</v>
+        <v>-1983193.86105263</v>
       </c>
       <c r="F7" s="20"/>
     </row>
@@ -3737,7 +4030,7 @@
       <c r="D9" s="20"/>
       <c r="E9" s="24" t="n">
         <f aca="false">Consolidated!N26</f>
-        <v>2778660.99438651</v>
+        <v>2770260.99438651</v>
       </c>
       <c r="F9" s="20"/>
     </row>
@@ -3747,7 +4040,7 @@
       </c>
       <c r="E10" s="25" t="n">
         <f aca="false">MIN(Consolidated!B38:M38)</f>
-        <v>-71258.4815801905</v>
+        <v>-77202.1815801902</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>57</v>
@@ -3759,7 +4052,7 @@
       </c>
       <c r="E11" s="25" t="n">
         <f aca="false">Consolidated!M38</f>
-        <v>1461018.76802361</v>
+        <v>1451575.06802361</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8808,6 +9101,1768 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:V47"/>
+  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="5" style="0" width="8.5"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="44" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="45" t="s">
+        <v>267</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="45"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="46" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="47" t="s">
+        <v>290</v>
+      </c>
+      <c r="B5" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="48" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="H5" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="L5" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="M5" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="N5" s="48" t="n">
+        <v>11</v>
+      </c>
+      <c r="O5" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="P5" s="48" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q5" s="48" t="n">
+        <v>13</v>
+      </c>
+      <c r="R5" s="48" t="n">
+        <v>13</v>
+      </c>
+      <c r="S5" s="48" t="n">
+        <v>13</v>
+      </c>
+      <c r="T5" s="48" t="n">
+        <v>14</v>
+      </c>
+      <c r="U5" s="48" t="n">
+        <v>13</v>
+      </c>
+      <c r="V5" s="48" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="49" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="50" t="s">
+        <v>292</v>
+      </c>
+      <c r="B8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="S8" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="T8" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="U8" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="V8" s="51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="52" t="s">
+        <v>293</v>
+      </c>
+      <c r="B9" s="53" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C9" s="53" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D9" s="53" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E9" s="53" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F9" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H9" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I9" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J9" s="53" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K9" s="53" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="L9" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" s="53" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="P9" s="53" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="Q9" s="53" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="R9" s="53" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S9" s="53" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="T9" s="53" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="U9" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="V9" s="53" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="50" t="s">
+        <v>294</v>
+      </c>
+      <c r="B10" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="P10" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="S10" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="T10" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="U10" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="V10" s="51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="52" t="s">
+        <v>293</v>
+      </c>
+      <c r="B11" s="53" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C11" s="53" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="D11" s="53" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E11" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="53" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G11" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K11" s="53" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L11" s="53" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M11" s="53" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="N11" s="53" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O11" s="53" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="P11" s="53" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="Q11" s="53" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="R11" s="53" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="S11" s="53" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="T11" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="U11" s="53" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="V11" s="53" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="50" t="s">
+        <v>295</v>
+      </c>
+      <c r="B12" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="H12" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="I12" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="J12" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="K12" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="L12" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="M12" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="N12" s="51" t="n">
+        <v>9</v>
+      </c>
+      <c r="O12" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="P12" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q12" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="R12" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="S12" s="51" t="n">
+        <v>12</v>
+      </c>
+      <c r="T12" s="51" t="n">
+        <v>13</v>
+      </c>
+      <c r="U12" s="51" t="n">
+        <v>13</v>
+      </c>
+      <c r="V12" s="51" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="52" t="s">
+        <v>293</v>
+      </c>
+      <c r="B13" s="53" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="C13" s="53" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="D13" s="53" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="E13" s="53" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F13" s="53" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G13" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="I13" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="J13" s="53" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="K13" s="53" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="L13" s="53" t="n">
+        <v>8.8</v>
+      </c>
+      <c r="M13" s="53" t="n">
+        <v>8.8</v>
+      </c>
+      <c r="N13" s="53" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="O13" s="53" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="P13" s="53" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="Q13" s="53" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="R13" s="53" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="S13" s="53" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="T13" s="53" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="U13" s="53" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="V13" s="53" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="B14" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="M14" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="N14" s="51" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" s="51" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q14" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="R14" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="S14" s="51" t="n">
+        <v>7</v>
+      </c>
+      <c r="T14" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="U14" s="51" t="n">
+        <v>8</v>
+      </c>
+      <c r="V14" s="51" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="52" t="s">
+        <v>293</v>
+      </c>
+      <c r="B15" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C15" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="D15" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E15" s="53" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F15" s="53" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G15" s="53" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H15" s="53" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="I15" s="53" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="J15" s="53" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="K15" s="53" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="L15" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="M15" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="N15" s="53" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O15" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="53" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="Q15" s="53" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="R15" s="53" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="S15" s="53" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="T15" s="53" t="n">
+        <v>8.7</v>
+      </c>
+      <c r="U15" s="53" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="V15" s="53" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="50" t="s">
+        <v>297</v>
+      </c>
+      <c r="B16" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="I16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="P16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="R16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="S16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="T16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="U16" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="V16" s="51" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="B17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="H17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="M17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="N17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="O17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="P17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="R17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="S17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="T17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="U17" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="V17" s="51" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="50" t="s">
+        <v>299</v>
+      </c>
+      <c r="B18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="G18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="J18" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="N18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="O18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="P18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="R18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="S18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="T18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="U18" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="V18" s="51" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="54" t="s">
+        <v>300</v>
+      </c>
+      <c r="B19" s="55" t="n">
+        <f aca="false">B8+B10+B12+B14+B16+B17+B18</f>
+        <v>17</v>
+      </c>
+      <c r="C19" s="55" t="n">
+        <f aca="false">C8+C10+C12+C14+C16+C17+C18</f>
+        <v>19</v>
+      </c>
+      <c r="D19" s="55" t="n">
+        <f aca="false">D8+D10+D12+D14+D16+D17+D18</f>
+        <v>22</v>
+      </c>
+      <c r="E19" s="55" t="n">
+        <f aca="false">E8+E10+E12+E14+E16+E17+E18</f>
+        <v>23</v>
+      </c>
+      <c r="F19" s="55" t="n">
+        <f aca="false">F8+F10+F12+F14+F16+F17+F18</f>
+        <v>23</v>
+      </c>
+      <c r="G19" s="55" t="n">
+        <f aca="false">G8+G10+G12+G14+G16+G17+G18</f>
+        <v>25</v>
+      </c>
+      <c r="H19" s="55" t="n">
+        <f aca="false">H8+H10+H12+H14+H16+H17+H18</f>
+        <v>26</v>
+      </c>
+      <c r="I19" s="55" t="n">
+        <f aca="false">I8+I10+I12+I14+I16+I17+I18</f>
+        <v>26</v>
+      </c>
+      <c r="J19" s="55" t="n">
+        <f aca="false">J8+J10+J12+J14+J16+J17+J18</f>
+        <v>27</v>
+      </c>
+      <c r="K19" s="55" t="n">
+        <f aca="false">K8+K10+K12+K14+K16+K17+K18</f>
+        <v>26</v>
+      </c>
+      <c r="L19" s="55" t="n">
+        <f aca="false">L8+L10+L12+L14+L16+L17+L18</f>
+        <v>27</v>
+      </c>
+      <c r="M19" s="55" t="n">
+        <f aca="false">M8+M10+M12+M14+M16+M17+M18</f>
+        <v>27</v>
+      </c>
+      <c r="N19" s="55" t="n">
+        <f aca="false">N8+N10+N12+N14+N16+N17+N18</f>
+        <v>28</v>
+      </c>
+      <c r="O19" s="55" t="n">
+        <f aca="false">O8+O10+O12+O14+O16+O17+O18</f>
+        <v>30</v>
+      </c>
+      <c r="P19" s="55" t="n">
+        <f aca="false">P8+P10+P12+P14+P16+P17+P18</f>
+        <v>34</v>
+      </c>
+      <c r="Q19" s="55" t="n">
+        <f aca="false">Q8+Q10+Q12+Q14+Q16+Q17+Q18</f>
+        <v>34</v>
+      </c>
+      <c r="R19" s="55" t="n">
+        <f aca="false">R8+R10+R12+R14+R16+R17+R18</f>
+        <v>34</v>
+      </c>
+      <c r="S19" s="55" t="n">
+        <f aca="false">S8+S10+S12+S14+S16+S17+S18</f>
+        <v>34</v>
+      </c>
+      <c r="T19" s="55" t="n">
+        <f aca="false">T8+T10+T12+T14+T16+T17+T18</f>
+        <v>38</v>
+      </c>
+      <c r="U19" s="55" t="n">
+        <f aca="false">U8+U10+U12+U14+U16+U17+U18</f>
+        <v>38</v>
+      </c>
+      <c r="V19" s="55" t="n">
+        <f aca="false">V8+V10+V12+V14+V16+V17+V18</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="52" t="s">
+        <v>301</v>
+      </c>
+      <c r="B20" s="56"/>
+      <c r="C20" s="56" t="n">
+        <f aca="false">C19-B19</f>
+        <v>2</v>
+      </c>
+      <c r="D20" s="56" t="n">
+        <f aca="false">D19-C19</f>
+        <v>3</v>
+      </c>
+      <c r="E20" s="56" t="n">
+        <f aca="false">E19-D19</f>
+        <v>1</v>
+      </c>
+      <c r="F20" s="56" t="n">
+        <f aca="false">F19-E19</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="56" t="n">
+        <f aca="false">G19-F19</f>
+        <v>2</v>
+      </c>
+      <c r="H20" s="56" t="n">
+        <f aca="false">H19-G19</f>
+        <v>1</v>
+      </c>
+      <c r="I20" s="56" t="n">
+        <f aca="false">I19-H19</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="56" t="n">
+        <f aca="false">J19-I19</f>
+        <v>1</v>
+      </c>
+      <c r="K20" s="56" t="n">
+        <f aca="false">K19-J19</f>
+        <v>-1</v>
+      </c>
+      <c r="L20" s="56" t="n">
+        <f aca="false">L19-K19</f>
+        <v>1</v>
+      </c>
+      <c r="M20" s="56" t="n">
+        <f aca="false">M19-L19</f>
+        <v>0</v>
+      </c>
+      <c r="N20" s="56" t="n">
+        <f aca="false">N19-M19</f>
+        <v>1</v>
+      </c>
+      <c r="O20" s="56" t="n">
+        <f aca="false">O19-N19</f>
+        <v>2</v>
+      </c>
+      <c r="P20" s="56" t="n">
+        <f aca="false">P19-O19</f>
+        <v>4</v>
+      </c>
+      <c r="Q20" s="56" t="n">
+        <f aca="false">Q19-P19</f>
+        <v>0</v>
+      </c>
+      <c r="R20" s="56" t="n">
+        <f aca="false">R19-Q19</f>
+        <v>0</v>
+      </c>
+      <c r="S20" s="56" t="n">
+        <f aca="false">S19-R19</f>
+        <v>0</v>
+      </c>
+      <c r="T20" s="56" t="n">
+        <f aca="false">T19-S19</f>
+        <v>4</v>
+      </c>
+      <c r="U20" s="56" t="n">
+        <f aca="false">U19-T19</f>
+        <v>0</v>
+      </c>
+      <c r="V20" s="56" t="n">
+        <f aca="false">V19-U19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="50" t="s">
+        <v>302</v>
+      </c>
+      <c r="B22" s="51" t="n">
+        <v>187694</v>
+      </c>
+      <c r="C22" s="51" t="n">
+        <v>295949</v>
+      </c>
+      <c r="D22" s="51" t="n">
+        <v>198646</v>
+      </c>
+      <c r="E22" s="51" t="n">
+        <v>215852</v>
+      </c>
+      <c r="F22" s="51" t="n">
+        <v>217611</v>
+      </c>
+      <c r="G22" s="51" t="n">
+        <v>223657</v>
+      </c>
+      <c r="H22" s="51" t="n">
+        <v>267964</v>
+      </c>
+      <c r="I22" s="51" t="n">
+        <v>267964</v>
+      </c>
+      <c r="J22" s="51" t="n">
+        <v>356298</v>
+      </c>
+      <c r="K22" s="51" t="n">
+        <v>270881</v>
+      </c>
+      <c r="L22" s="51" t="n">
+        <v>281298</v>
+      </c>
+      <c r="M22" s="51" t="n">
+        <v>281298</v>
+      </c>
+      <c r="N22" s="51" t="n">
+        <v>294631</v>
+      </c>
+      <c r="O22" s="51" t="n">
+        <v>318381</v>
+      </c>
+      <c r="P22" s="51" t="n">
+        <v>366298</v>
+      </c>
+      <c r="Q22" s="51" t="n">
+        <v>366298</v>
+      </c>
+      <c r="R22" s="51" t="n">
+        <v>366298</v>
+      </c>
+      <c r="S22" s="51" t="n">
+        <v>366298</v>
+      </c>
+      <c r="T22" s="51" t="n">
+        <v>415881</v>
+      </c>
+      <c r="U22" s="51" t="n">
+        <v>415881</v>
+      </c>
+      <c r="V22" s="51" t="n">
+        <v>615881</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="57" t="s">
+        <v>303</v>
+      </c>
+      <c r="B23" s="58" t="n">
+        <f aca="false">B22/B5</f>
+        <v>37538.8</v>
+      </c>
+      <c r="C23" s="58" t="n">
+        <f aca="false">C22/C5</f>
+        <v>59189.8</v>
+      </c>
+      <c r="D23" s="58" t="n">
+        <f aca="false">D22/D5</f>
+        <v>39729.2</v>
+      </c>
+      <c r="E23" s="58" t="n">
+        <f aca="false">E22/E5</f>
+        <v>43170.4</v>
+      </c>
+      <c r="F23" s="58" t="n">
+        <f aca="false">F22/F5</f>
+        <v>31087.2857142857</v>
+      </c>
+      <c r="G23" s="58" t="n">
+        <f aca="false">G22/G5</f>
+        <v>27957.125</v>
+      </c>
+      <c r="H23" s="58" t="n">
+        <f aca="false">H22/H5</f>
+        <v>33495.5</v>
+      </c>
+      <c r="I23" s="58" t="n">
+        <f aca="false">I22/I5</f>
+        <v>33495.5</v>
+      </c>
+      <c r="J23" s="58" t="n">
+        <f aca="false">J22/J5</f>
+        <v>44537.25</v>
+      </c>
+      <c r="K23" s="58" t="n">
+        <f aca="false">K22/K5</f>
+        <v>30097.8888888889</v>
+      </c>
+      <c r="L23" s="58" t="n">
+        <f aca="false">L22/L5</f>
+        <v>28129.8</v>
+      </c>
+      <c r="M23" s="58" t="n">
+        <f aca="false">M22/M5</f>
+        <v>28129.8</v>
+      </c>
+      <c r="N23" s="58" t="n">
+        <f aca="false">N22/N5</f>
+        <v>26784.6363636364</v>
+      </c>
+      <c r="O23" s="58" t="n">
+        <f aca="false">O22/O5</f>
+        <v>26531.75</v>
+      </c>
+      <c r="P23" s="58" t="n">
+        <f aca="false">P22/P5</f>
+        <v>26164.1428571429</v>
+      </c>
+      <c r="Q23" s="58" t="n">
+        <f aca="false">Q22/Q5</f>
+        <v>28176.7692307692</v>
+      </c>
+      <c r="R23" s="58" t="n">
+        <f aca="false">R22/R5</f>
+        <v>28176.7692307692</v>
+      </c>
+      <c r="S23" s="58" t="n">
+        <f aca="false">S22/S5</f>
+        <v>28176.7692307692</v>
+      </c>
+      <c r="T23" s="58" t="n">
+        <f aca="false">T22/T5</f>
+        <v>29705.7857142857</v>
+      </c>
+      <c r="U23" s="58" t="n">
+        <f aca="false">U22/U5</f>
+        <v>31990.8461538462</v>
+      </c>
+      <c r="V23" s="58" t="n">
+        <f aca="false">V22/V5</f>
+        <v>47375.4615384615</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="57" t="s">
+        <v>304</v>
+      </c>
+      <c r="B24" s="59" t="n">
+        <f aca="false">B5/B8</f>
+        <v>1.66666666666667</v>
+      </c>
+      <c r="C24" s="59" t="n">
+        <f aca="false">C5/C8</f>
+        <v>1.66666666666667</v>
+      </c>
+      <c r="D24" s="59" t="n">
+        <f aca="false">D5/D8</f>
+        <v>1.66666666666667</v>
+      </c>
+      <c r="E24" s="59" t="n">
+        <f aca="false">E5/E8</f>
+        <v>1.66666666666667</v>
+      </c>
+      <c r="F24" s="59" t="n">
+        <f aca="false">F5/F8</f>
+        <v>2.33333333333333</v>
+      </c>
+      <c r="G24" s="59" t="n">
+        <f aca="false">G5/G8</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="H24" s="59" t="n">
+        <f aca="false">H5/H8</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="I24" s="59" t="n">
+        <f aca="false">I5/I8</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="J24" s="59" t="n">
+        <f aca="false">J5/J8</f>
+        <v>2.66666666666667</v>
+      </c>
+      <c r="K24" s="59" t="n">
+        <f aca="false">K5/K8</f>
+        <v>3</v>
+      </c>
+      <c r="L24" s="59" t="n">
+        <f aca="false">L5/L8</f>
+        <v>3.33333333333333</v>
+      </c>
+      <c r="M24" s="59" t="n">
+        <f aca="false">M5/M8</f>
+        <v>3.33333333333333</v>
+      </c>
+      <c r="N24" s="59" t="n">
+        <f aca="false">N5/N8</f>
+        <v>3.66666666666667</v>
+      </c>
+      <c r="O24" s="59" t="n">
+        <f aca="false">O5/O8</f>
+        <v>4</v>
+      </c>
+      <c r="P24" s="59" t="n">
+        <f aca="false">P5/P8</f>
+        <v>4.66666666666667</v>
+      </c>
+      <c r="Q24" s="59" t="n">
+        <f aca="false">Q5/Q8</f>
+        <v>4.33333333333333</v>
+      </c>
+      <c r="R24" s="59" t="n">
+        <f aca="false">R5/R8</f>
+        <v>4.33333333333333</v>
+      </c>
+      <c r="S24" s="59" t="n">
+        <f aca="false">S5/S8</f>
+        <v>4.33333333333333</v>
+      </c>
+      <c r="T24" s="59" t="n">
+        <f aca="false">T5/T8</f>
+        <v>3.5</v>
+      </c>
+      <c r="U24" s="59" t="n">
+        <f aca="false">U5/U8</f>
+        <v>3.25</v>
+      </c>
+      <c r="V24" s="59" t="n">
+        <f aca="false">V5/V8</f>
+        <v>3.25</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="60" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="46" t="s">
+        <v>306</v>
+      </c>
+      <c r="B27" s="46" t="s">
+        <v>307</v>
+      </c>
+      <c r="C27" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="D27" s="46" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="57" t="s">
+        <v>310</v>
+      </c>
+      <c r="B28" s="59" t="n">
+        <f aca="false">AVERAGE(B5:J5)</f>
+        <v>6.55555555555556</v>
+      </c>
+      <c r="C28" s="59" t="n">
+        <f aca="false">AVERAGE(K5:V5)</f>
+        <v>12.0833333333333</v>
+      </c>
+      <c r="D28" s="59" t="n">
+        <f aca="false">C28-B28</f>
+        <v>5.52777777777778</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="57" t="s">
+        <v>311</v>
+      </c>
+      <c r="B29" s="58" t="n">
+        <f aca="false">J5</f>
+        <v>8</v>
+      </c>
+      <c r="C29" s="58" t="n">
+        <f aca="false">V5</f>
+        <v>13</v>
+      </c>
+      <c r="D29" s="58" t="n">
+        <f aca="false">C29-B29</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="57" t="s">
+        <v>312</v>
+      </c>
+      <c r="B30" s="59" t="n">
+        <f aca="false">AVERAGE(B19:J19)</f>
+        <v>23.1111111111111</v>
+      </c>
+      <c r="C30" s="59" t="n">
+        <f aca="false">AVERAGE(K19:V19)</f>
+        <v>32.3333333333333</v>
+      </c>
+      <c r="D30" s="59" t="n">
+        <f aca="false">C30-B30</f>
+        <v>9.22222222222223</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="57" t="s">
+        <v>313</v>
+      </c>
+      <c r="B31" s="58" t="n">
+        <f aca="false">J19</f>
+        <v>27</v>
+      </c>
+      <c r="C31" s="58" t="n">
+        <f aca="false">V19</f>
+        <v>38</v>
+      </c>
+      <c r="D31" s="58" t="n">
+        <f aca="false">C31-B31</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="57" t="s">
+        <v>314</v>
+      </c>
+      <c r="B32" s="58" t="n">
+        <f aca="false">J8</f>
+        <v>3</v>
+      </c>
+      <c r="C32" s="58" t="n">
+        <f aca="false">V8</f>
+        <v>4</v>
+      </c>
+      <c r="D32" s="58" t="n">
+        <f aca="false">C32-B32</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="57" t="s">
+        <v>315</v>
+      </c>
+      <c r="B33" s="58" t="n">
+        <f aca="false">J10</f>
+        <v>2</v>
+      </c>
+      <c r="C33" s="58" t="n">
+        <f aca="false">V10</f>
+        <v>4</v>
+      </c>
+      <c r="D33" s="58" t="n">
+        <f aca="false">C33-B33</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="57" t="s">
+        <v>316</v>
+      </c>
+      <c r="B34" s="58" t="n">
+        <f aca="false">J12</f>
+        <v>8</v>
+      </c>
+      <c r="C34" s="58" t="n">
+        <f aca="false">V12</f>
+        <v>13</v>
+      </c>
+      <c r="D34" s="58" t="n">
+        <f aca="false">C34-B34</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="57" t="s">
+        <v>317</v>
+      </c>
+      <c r="B35" s="58" t="n">
+        <f aca="false">J14</f>
+        <v>4</v>
+      </c>
+      <c r="C35" s="58" t="n">
+        <f aca="false">V14</f>
+        <v>8</v>
+      </c>
+      <c r="D35" s="58" t="n">
+        <f aca="false">C35-B35</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="57" t="s">
+        <v>318</v>
+      </c>
+      <c r="B36" s="58" t="n">
+        <f aca="false">J16</f>
+        <v>3</v>
+      </c>
+      <c r="C36" s="58" t="n">
+        <f aca="false">V16</f>
+        <v>3</v>
+      </c>
+      <c r="D36" s="58" t="n">
+        <f aca="false">C36-B36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="57" t="s">
+        <v>319</v>
+      </c>
+      <c r="B37" s="58" t="n">
+        <f aca="false">J17</f>
+        <v>4</v>
+      </c>
+      <c r="C37" s="58" t="n">
+        <f aca="false">V17</f>
+        <v>4</v>
+      </c>
+      <c r="D37" s="58" t="n">
+        <f aca="false">C37-B37</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="57" t="s">
+        <v>320</v>
+      </c>
+      <c r="B38" s="58" t="n">
+        <f aca="false">J18</f>
+        <v>3</v>
+      </c>
+      <c r="C38" s="58" t="n">
+        <f aca="false">V18</f>
+        <v>2</v>
+      </c>
+      <c r="D38" s="58" t="n">
+        <f aca="false">C38-B38</f>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="57" t="s">
+        <v>321</v>
+      </c>
+      <c r="B39" s="61" t="n">
+        <f aca="false">AVERAGE(B5:J5)/AVERAGE(B8:J8)</f>
+        <v>2.18518518518519</v>
+      </c>
+      <c r="C39" s="61" t="n">
+        <f aca="false">AVERAGE(K5:V5)/AVERAGE(K8:V8)</f>
+        <v>3.71794871794872</v>
+      </c>
+      <c r="D39" s="61" t="n">
+        <f aca="false">C39-B39</f>
+        <v>1.53276353276353</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="57" t="s">
+        <v>322</v>
+      </c>
+      <c r="B40" s="62" t="n">
+        <f aca="false">AVERAGE(B5:J5)/AVERAGE(B12:J12)</f>
+        <v>1.07272727272727</v>
+      </c>
+      <c r="C40" s="62" t="n">
+        <f aca="false">AVERAGE(K5:V5)/AVERAGE(K12:V12)</f>
+        <v>1.11538461538462</v>
+      </c>
+      <c r="D40" s="62" t="n">
+        <f aca="false">C40-B40</f>
+        <v>0.0426573426573427</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="57" t="s">
+        <v>323</v>
+      </c>
+      <c r="B41" s="58" t="n">
+        <f aca="false">SUM(B22:J22)/SUM(B5:J5)</f>
+        <v>37824.3220338983</v>
+      </c>
+      <c r="C41" s="58" t="n">
+        <f aca="false">SUM(K22:V22)/SUM(K5:V5)</f>
+        <v>30064.3034482759</v>
+      </c>
+      <c r="D41" s="58" t="n">
+        <f aca="false">C41-B41</f>
+        <v>-7760.01858562245</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="33" t="s">
+        <v>324</v>
+      </c>
+      <c r="B43" s="33"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="33"/>
+      <c r="E43" s="33"/>
+      <c r="F43" s="33"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="33"/>
+      <c r="I43" s="33"/>
+      <c r="J43" s="33"/>
+      <c r="K43" s="33"/>
+      <c r="L43" s="33"/>
+      <c r="M43" s="33"/>
+      <c r="N43" s="33"/>
+      <c r="O43" s="33"/>
+      <c r="P43" s="33"/>
+      <c r="Q43" s="33"/>
+      <c r="R43" s="33"/>
+      <c r="S43" s="33"/>
+      <c r="T43" s="33"/>
+      <c r="U43" s="33"/>
+      <c r="V43" s="33"/>
+    </row>
+    <row r="44" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="33" t="s">
+        <v>325</v>
+      </c>
+      <c r="B44" s="33"/>
+      <c r="C44" s="33"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="33"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="33"/>
+      <c r="I44" s="33"/>
+      <c r="J44" s="33"/>
+      <c r="K44" s="33"/>
+      <c r="L44" s="33"/>
+      <c r="M44" s="33"/>
+      <c r="N44" s="33"/>
+      <c r="O44" s="33"/>
+      <c r="P44" s="33"/>
+      <c r="Q44" s="33"/>
+      <c r="R44" s="33"/>
+      <c r="S44" s="33"/>
+      <c r="T44" s="33"/>
+      <c r="U44" s="33"/>
+      <c r="V44" s="33"/>
+    </row>
+    <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="33" t="s">
+        <v>326</v>
+      </c>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="33"/>
+      <c r="I45" s="33"/>
+      <c r="J45" s="33"/>
+      <c r="K45" s="33"/>
+      <c r="L45" s="33"/>
+      <c r="M45" s="33"/>
+      <c r="N45" s="33"/>
+      <c r="O45" s="33"/>
+      <c r="P45" s="33"/>
+      <c r="Q45" s="33"/>
+      <c r="R45" s="33"/>
+      <c r="S45" s="33"/>
+      <c r="T45" s="33"/>
+      <c r="U45" s="33"/>
+      <c r="V45" s="33"/>
+    </row>
+    <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="33"/>
+      <c r="H46" s="33"/>
+      <c r="I46" s="33"/>
+      <c r="J46" s="33"/>
+      <c r="K46" s="33"/>
+      <c r="L46" s="33"/>
+      <c r="M46" s="33"/>
+      <c r="N46" s="33"/>
+      <c r="O46" s="33"/>
+      <c r="P46" s="33"/>
+      <c r="Q46" s="33"/>
+      <c r="R46" s="33"/>
+      <c r="S46" s="33"/>
+      <c r="T46" s="33"/>
+      <c r="U46" s="33"/>
+      <c r="V46" s="33"/>
+    </row>
+    <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="33" t="s">
+        <v>328</v>
+      </c>
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="33"/>
+      <c r="K47" s="33"/>
+      <c r="L47" s="33"/>
+      <c r="M47" s="33"/>
+      <c r="N47" s="33"/>
+      <c r="O47" s="33"/>
+      <c r="P47" s="33"/>
+      <c r="Q47" s="33"/>
+      <c r="R47" s="33"/>
+      <c r="S47" s="33"/>
+      <c r="T47" s="33"/>
+      <c r="U47" s="33"/>
+      <c r="V47" s="33"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A43:V43"/>
+    <mergeCell ref="A44:V44"/>
+    <mergeCell ref="A45:V45"/>
+    <mergeCell ref="A46:V46"/>
+    <mergeCell ref="A47:V47"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:N60"/>
   <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -8820,7 +10875,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>266</v>
+        <v>329</v>
       </c>
       <c r="B1" s="36"/>
       <c r="C1" s="36"/>
@@ -8838,7 +10893,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>267</v>
+        <v>330</v>
       </c>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
@@ -8934,7 +10989,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="38" t="s">
-        <v>268</v>
+        <v>331</v>
       </c>
       <c r="B6" s="39" t="n">
         <v>23906.25</v>
@@ -8979,7 +11034,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="38" t="s">
-        <v>269</v>
+        <v>332</v>
       </c>
       <c r="B7" s="39" t="n">
         <v>0</v>
@@ -9024,52 +11079,52 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>270</v>
+        <v>333</v>
       </c>
       <c r="B8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="C8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="D8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="E8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="F8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="G8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="H8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="I8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="J8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="K8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="L8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="M8" s="39" t="n">
-        <v>9500</v>
+        <v>8800</v>
       </c>
       <c r="N8" s="40" t="n">
         <f aca="false">SUM(B8:M8)</f>
-        <v>114000</v>
+        <v>105600</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>271</v>
+        <v>334</v>
       </c>
       <c r="B9" s="39" t="n">
         <v>0</v>
@@ -9114,7 +11169,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="38" t="s">
-        <v>272</v>
+        <v>335</v>
       </c>
       <c r="B10" s="39" t="n">
         <v>3157.89473684211</v>
@@ -9159,59 +11214,59 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>273</v>
+        <v>336</v>
       </c>
       <c r="B11" s="40" t="n">
         <f aca="false">B6+B7+B8+B9+B10</f>
-        <v>36564.1447368421</v>
+        <v>35864.1447368421</v>
       </c>
       <c r="C11" s="40" t="n">
         <f aca="false">C6+C7+C8+C9+C10</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="D11" s="40" t="n">
         <f aca="false">D6+D7+D8+D9+D10</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="E11" s="40" t="n">
         <f aca="false">E6+E7+E8+E9+E10</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="F11" s="40" t="n">
         <f aca="false">F6+F7+F8+F9+F10</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="G11" s="40" t="n">
         <f aca="false">G6+G7+G8+G9+G10</f>
-        <v>39722.0394736842</v>
+        <v>39022.0394736842</v>
       </c>
       <c r="H11" s="40" t="n">
         <f aca="false">H6+H7+H8+H9+H10</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="I11" s="40" t="n">
         <f aca="false">I6+I7+I8+I9+I10</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="J11" s="40" t="n">
         <f aca="false">J6+J7+J8+J9+J10</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="K11" s="40" t="n">
         <f aca="false">K6+K7+K8+K9+K10</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="L11" s="40" t="n">
         <f aca="false">L6+L7+L8+L9+L10</f>
-        <v>15815.7894736842</v>
+        <v>15115.7894736842</v>
       </c>
       <c r="M11" s="40" t="n">
         <f aca="false">M6+M7+M8+M9+M10</f>
-        <v>73190.7894736842</v>
+        <v>72490.7894736842</v>
       </c>
       <c r="N11" s="40" t="n">
         <f aca="false">N6+N7+N8+N9+N10</f>
-        <v>387444.078947369</v>
+        <v>379044.078947369</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9594,7 +11649,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="38" t="s">
-        <v>274</v>
+        <v>337</v>
       </c>
       <c r="B21" s="39" t="n">
         <v>-290</v>
@@ -9639,7 +11694,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="38" t="s">
-        <v>275</v>
+        <v>338</v>
       </c>
       <c r="B22" s="39" t="n">
         <v>-245</v>
@@ -9684,7 +11739,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="38" t="s">
-        <v>276</v>
+        <v>339</v>
       </c>
       <c r="B23" s="39" t="n">
         <v>-1179.5</v>
@@ -9729,7 +11784,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="38" t="s">
-        <v>277</v>
+        <v>340</v>
       </c>
       <c r="B24" s="39" t="n">
         <v>-366.3</v>
@@ -9774,7 +11829,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="38" t="s">
-        <v>278</v>
+        <v>341</v>
       </c>
       <c r="B25" s="39" t="n">
         <v>-50.07</v>
@@ -9999,7 +12054,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="38" t="s">
-        <v>279</v>
+        <v>342</v>
       </c>
       <c r="B30" s="39" t="n">
         <v>-1586.17</v>
@@ -10044,7 +12099,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="38" t="s">
-        <v>280</v>
+        <v>343</v>
       </c>
       <c r="B31" s="39" t="n">
         <v>-3333.33</v>
@@ -10089,7 +12144,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="38" t="s">
-        <v>281</v>
+        <v>344</v>
       </c>
       <c r="B32" s="39" t="n">
         <v>-1905.31</v>
@@ -10134,7 +12189,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="38" t="s">
-        <v>282</v>
+        <v>345</v>
       </c>
       <c r="B33" s="39" t="n">
         <v>-2100</v>
@@ -10179,7 +12234,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="38" t="s">
-        <v>283</v>
+        <v>346</v>
       </c>
       <c r="B34" s="39" t="n">
         <v>-66666.6666666667</v>
@@ -10314,7 +12369,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="41" t="s">
-        <v>284</v>
+        <v>347</v>
       </c>
       <c r="B37" s="40" t="n">
         <f aca="false">B13+B14+B15+B16+B17+B18+B19+B20+B21+B22+B23+B24+B25+B26+B27+B28+B29+B30+B31+B32+B33+B34+B35+B36</f>
@@ -10371,59 +12426,59 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="42" t="s">
-        <v>285</v>
+        <v>348</v>
       </c>
       <c r="B38" s="43" t="n">
         <f aca="false">B11+B37</f>
-        <v>-163059.850263158</v>
+        <v>-163759.850263158</v>
       </c>
       <c r="C38" s="43" t="n">
         <f aca="false">C11+C37</f>
-        <v>-158151.955526316</v>
+        <v>-158851.955526316</v>
       </c>
       <c r="D38" s="43" t="n">
         <f aca="false">D11+D37</f>
-        <v>-158151.955526316</v>
+        <v>-158851.955526316</v>
       </c>
       <c r="E38" s="43" t="n">
         <f aca="false">E11+E37</f>
-        <v>-158151.955526316</v>
+        <v>-158851.955526316</v>
       </c>
       <c r="F38" s="43" t="n">
         <f aca="false">F11+F37</f>
-        <v>-156401.955526316</v>
+        <v>-157101.955526316</v>
       </c>
       <c r="G38" s="43" t="n">
         <f aca="false">G11+G37</f>
-        <v>-156401.955526316</v>
+        <v>-157101.955526316</v>
       </c>
       <c r="H38" s="43" t="n">
         <f aca="false">H11+H37</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="I38" s="43" t="n">
         <f aca="false">I11+I37</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="J38" s="43" t="n">
         <f aca="false">J11+J37</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="K38" s="43" t="n">
         <f aca="false">K11+K37</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="L38" s="43" t="n">
         <f aca="false">L11+L37</f>
-        <v>-180308.205526316</v>
+        <v>-181008.205526316</v>
       </c>
       <c r="M38" s="43" t="n">
         <f aca="false">M11+M37</f>
-        <v>-122933.205526316</v>
+        <v>-123633.205526316</v>
       </c>
       <c r="N38" s="43" t="n">
         <f aca="false">N11+N37</f>
-        <v>-1974793.86105263</v>
+        <v>-1983193.86105263</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -10457,7 +12512,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -10473,7 +12528,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>286</v>
+        <v>349</v>
       </c>
       <c r="B1" s="36"/>
       <c r="C1" s="36"/>
@@ -10491,7 +12546,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>287</v>
+        <v>350</v>
       </c>
       <c r="B2" s="36"/>
       <c r="C2" s="36"/>
@@ -10569,7 +12624,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>288</v>
+        <v>351</v>
       </c>
       <c r="B5" s="37"/>
       <c r="C5" s="37"/>
@@ -10587,7 +12642,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="38" t="s">
-        <v>289</v>
+        <v>352</v>
       </c>
       <c r="B6" s="39" t="n">
         <v>0</v>
@@ -10632,7 +12687,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="38" t="s">
-        <v>290</v>
+        <v>353</v>
       </c>
       <c r="B7" s="39" t="n">
         <v>0</v>
@@ -10677,7 +12732,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="41" t="s">
-        <v>291</v>
+        <v>354</v>
       </c>
       <c r="B8" s="40" t="n">
         <f aca="false">B6+B7</f>
@@ -10734,7 +12789,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="38" t="s">
-        <v>292</v>
+        <v>355</v>
       </c>
       <c r="B9" s="39" t="n">
         <v>0</v>
@@ -10779,7 +12834,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="42" t="s">
-        <v>293</v>
+        <v>356</v>
       </c>
       <c r="B10" s="43" t="n">
         <f aca="false">B8+B9</f>
@@ -10852,7 +12907,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>294</v>
+        <v>357</v>
       </c>
       <c r="B12" s="37"/>
       <c r="C12" s="37"/>
@@ -11005,7 +13060,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="38" t="s">
-        <v>295</v>
+        <v>358</v>
       </c>
       <c r="B16" s="39" t="n">
         <v>9750</v>
@@ -11050,7 +13105,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="41" t="s">
-        <v>296</v>
+        <v>359</v>
       </c>
       <c r="B17" s="40" t="n">
         <f aca="false">B13+B14+B15+B16</f>
@@ -11123,7 +13178,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>297</v>
+        <v>360</v>
       </c>
       <c r="B19" s="36"/>
       <c r="C19" s="36"/>
@@ -11141,7 +13196,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>298</v>
+        <v>361</v>
       </c>
       <c r="B20" s="36"/>
       <c r="C20" s="36"/>
@@ -11155,13 +13210,13 @@
       <c r="K20" s="36"/>
       <c r="L20" s="36"/>
       <c r="M20" s="36"/>
-      <c r="N20" s="44" t="n">
+      <c r="N20" s="63" t="n">
         <v>172240.34</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>299</v>
+        <v>362</v>
       </c>
       <c r="B21" s="36"/>
       <c r="C21" s="36"/>
@@ -11175,13 +13230,13 @@
       <c r="K21" s="36"/>
       <c r="L21" s="36"/>
       <c r="M21" s="36"/>
-      <c r="N21" s="44" t="n">
+      <c r="N21" s="63" t="n">
         <v>25000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>300</v>
+        <v>363</v>
       </c>
       <c r="B22" s="36"/>
       <c r="C22" s="36"/>
@@ -11195,13 +13250,13 @@
       <c r="K22" s="36"/>
       <c r="L22" s="36"/>
       <c r="M22" s="36"/>
-      <c r="N22" s="44" t="n">
+      <c r="N22" s="63" t="n">
         <v>150000</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>301</v>
+        <v>364</v>
       </c>
       <c r="B23" s="36"/>
       <c r="C23" s="36"/>
@@ -11215,13 +13270,13 @@
       <c r="K23" s="36"/>
       <c r="L23" s="36"/>
       <c r="M23" s="36"/>
-      <c r="N23" s="44" t="n">
+      <c r="N23" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>302</v>
+        <v>365</v>
       </c>
       <c r="B24" s="36"/>
       <c r="C24" s="36"/>
@@ -11235,13 +13290,13 @@
       <c r="K24" s="36"/>
       <c r="L24" s="36"/>
       <c r="M24" s="36"/>
-      <c r="N24" s="44" t="n">
+      <c r="N24" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>303</v>
+        <v>366</v>
       </c>
       <c r="B25" s="36"/>
       <c r="C25" s="36"/>
@@ -11255,13 +13310,13 @@
       <c r="K25" s="36"/>
       <c r="L25" s="36"/>
       <c r="M25" s="36"/>
-      <c r="N25" s="44" t="n">
+      <c r="N25" s="63" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>304</v>
+        <v>367</v>
       </c>
       <c r="B26" s="36"/>
       <c r="C26" s="36"/>
@@ -11275,13 +13330,13 @@
       <c r="K26" s="36"/>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
-      <c r="N26" s="44" t="n">
+      <c r="N26" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>305</v>
+        <v>368</v>
       </c>
       <c r="B27" s="36"/>
       <c r="C27" s="36"/>
@@ -11295,13 +13350,13 @@
       <c r="K27" s="36"/>
       <c r="L27" s="36"/>
       <c r="M27" s="36"/>
-      <c r="N27" s="44" t="n">
+      <c r="N27" s="63" t="n">
         <v>-3559.66000000002</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>306</v>
+        <v>369</v>
       </c>
       <c r="B28" s="36"/>
       <c r="C28" s="36"/>
@@ -11315,13 +13370,13 @@
       <c r="K28" s="36"/>
       <c r="L28" s="36"/>
       <c r="M28" s="36"/>
-      <c r="N28" s="44" t="n">
+      <c r="N28" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>307</v>
+        <v>370</v>
       </c>
       <c r="B29" s="36"/>
       <c r="C29" s="36"/>
@@ -11335,13 +13390,13 @@
       <c r="K29" s="36"/>
       <c r="L29" s="36"/>
       <c r="M29" s="36"/>
-      <c r="N29" s="44" t="n">
+      <c r="N29" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>308</v>
+        <v>371</v>
       </c>
       <c r="B30" s="36"/>
       <c r="C30" s="36"/>
@@ -11355,13 +13410,13 @@
       <c r="K30" s="36"/>
       <c r="L30" s="36"/>
       <c r="M30" s="36"/>
-      <c r="N30" s="44" t="n">
+      <c r="N30" s="63" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>309</v>
+        <v>372</v>
       </c>
       <c r="B31" s="36"/>
       <c r="C31" s="36"/>
@@ -11375,13 +13430,13 @@
       <c r="K31" s="36"/>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
-      <c r="N31" s="44" t="n">
+      <c r="N31" s="63" t="n">
         <v>3559.66000000002</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>310</v>
+        <v>373</v>
       </c>
       <c r="B32" s="36"/>
       <c r="C32" s="36"/>
@@ -11395,7 +13450,7 @@
       <c r="K32" s="36"/>
       <c r="L32" s="36"/>
       <c r="M32" s="36"/>
-      <c r="N32" s="44" t="n">
+      <c r="N32" s="63" t="n">
         <v>3559.66000000003</v>
       </c>
     </row>
@@ -11410,7 +13465,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -11424,40 +13479,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>311</v>
+        <v>374</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
-        <v>312</v>
-      </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
+      <c r="A2" s="64" t="s">
+        <v>375</v>
+      </c>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>313</v>
+        <v>376</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>314</v>
+        <v>377</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>315</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>316</v>
+        <v>379</v>
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">-'Six Peak'!N29*222000/337000</f>
         <v>222000</v>
       </c>
-      <c r="C5" s="46" t="n">
+      <c r="C5" s="65" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="9" t="n">
@@ -11467,13 +13522,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>317</v>
+        <v>380</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">-(('Six Peak'!N13+'Six Peak'!N14+'Six Peak'!N16+'Six Peak'!N17)*157500/657500+'Six Peak'!N15/3)</f>
         <v>221014.5</v>
       </c>
-      <c r="C6" s="46" t="n">
+      <c r="C6" s="65" t="n">
         <v>0.9</v>
       </c>
       <c r="D6" s="9" t="n">
@@ -11483,13 +13538,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>318</v>
+        <v>381</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">-(('Six Peak'!N13+'Six Peak'!N14+'Six Peak'!N16+'Six Peak'!N17)*250000/657500+'Six Peak'!N15/3)</f>
         <v>322302</v>
       </c>
-      <c r="C7" s="46" t="n">
+      <c r="C7" s="65" t="n">
         <v>0.75</v>
       </c>
       <c r="D7" s="9" t="n">
@@ -11499,13 +13554,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>319</v>
+        <v>382</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">-'Six Peak'!N34/2</f>
         <v>400000</v>
       </c>
-      <c r="C8" s="46" t="n">
+      <c r="C8" s="65" t="n">
         <v>0.5</v>
       </c>
       <c r="D8" s="9" t="n">
@@ -11515,13 +13570,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>320</v>
+        <v>383</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">-'Six Peak'!N34/2</f>
         <v>400000</v>
       </c>
-      <c r="C9" s="46" t="n">
+      <c r="C9" s="65" t="n">
         <v>0.1</v>
       </c>
       <c r="D9" s="9" t="n">
@@ -11531,13 +13586,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>321</v>
+        <v>384</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">-(('Six Peak'!N13+'Six Peak'!N14+'Six Peak'!N16+'Six Peak'!N17)*250000/657500+'Six Peak'!N15/3)</f>
         <v>322302</v>
       </c>
-      <c r="C10" s="46" t="n">
+      <c r="C10" s="65" t="n">
         <v>0.1</v>
       </c>
       <c r="D10" s="9" t="n">
@@ -11547,7 +13602,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>322</v>
+        <v>385</v>
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">SUM(B5:B10)</f>
@@ -11560,25 +13615,25 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="47" t="s">
-        <v>323</v>
-      </c>
-      <c r="B12" s="47"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
+      <c r="A12" s="66" t="s">
+        <v>386</v>
+      </c>
+      <c r="B12" s="66"/>
+      <c r="C12" s="66"/>
+      <c r="D12" s="66"/>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>324</v>
+        <v>387</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>325</v>
+        <v>388</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>326</v>
+        <v>389</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>327</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11604,7 +13659,7 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">Consolidated!N24</f>
-        <v>-1974793.86105263</v>
+        <v>-1983193.86105263</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">D11</f>
@@ -11612,7 +13667,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">B16+C16</f>
-        <v>-1039924.11105263</v>
+        <v>-1048324.11105263</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11633,11 +13688,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>328</v>
+        <v>391</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">SUM(B15:B17)</f>
-        <v>2778660.99438651</v>
+        <v>2770260.99438651</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">SUM(C15:C17)</f>
@@ -11645,7 +13700,7 @@
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">SUM(D15:D17)</f>
-        <v>2778660.99438651</v>
+        <v>2770260.99438651</v>
       </c>
     </row>
   </sheetData>
@@ -11663,7 +13718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -11677,7 +13732,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>329</v>
+        <v>392</v>
       </c>
       <c r="B1" s="36"/>
     </row>
@@ -11686,62 +13741,62 @@
       <c r="B2" s="36"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="48" t="s">
-        <v>330</v>
+      <c r="A3" s="67" t="s">
+        <v>393</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>331</v>
+        <v>394</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="48" t="s">
-        <v>332</v>
+      <c r="A4" s="67" t="s">
+        <v>395</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>333</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="48" t="s">
-        <v>334</v>
-      </c>
-      <c r="B5" s="49" t="n">
+      <c r="A5" s="67" t="s">
+        <v>397</v>
+      </c>
+      <c r="B5" s="68" t="n">
         <v>4752655</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="48" t="s">
-        <v>335</v>
-      </c>
-      <c r="B6" s="49" t="n">
-        <v>-1974794</v>
+      <c r="A6" s="67" t="s">
+        <v>398</v>
+      </c>
+      <c r="B6" s="68" t="n">
+        <v>-1983194</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="48" t="s">
-        <v>336</v>
-      </c>
-      <c r="B7" s="49"/>
+      <c r="A7" s="67" t="s">
+        <v>399</v>
+      </c>
+      <c r="B7" s="68"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="48" t="s">
-        <v>337</v>
-      </c>
-      <c r="B8" s="49" t="n">
+      <c r="A8" s="67" t="s">
+        <v>400</v>
+      </c>
+      <c r="B8" s="68" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="48" t="s">
-        <v>338</v>
-      </c>
-      <c r="B9" s="49" t="n">
-        <v>2778661</v>
+      <c r="A9" s="67" t="s">
+        <v>401</v>
+      </c>
+      <c r="B9" s="68" t="n">
+        <v>2770261</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="48" t="s">
-        <v>339</v>
+      <c r="A10" s="67" t="s">
+        <v>402</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">ROUND('Mgmt View (Hypothetical)'!C15+'Mgmt View (Hypothetical)'!C16,2)</f>
@@ -11749,8 +13804,8 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="48" t="s">
-        <v>340</v>
+      <c r="A11" s="67" t="s">
+        <v>403</v>
       </c>
       <c r="B11" s="1" t="n">
         <f aca="false">ROUND(Consolidated!N26-Consolidated!N11-Consolidated!N21,2)</f>
@@ -11759,47 +13814,47 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>341</v>
+        <v>404</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>342</v>
+        <v>405</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>343</v>
+        <v>406</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>344</v>
+        <v>407</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>345</v>
+        <v>408</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>346</v>
+        <v>409</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>347</v>
+        <v>410</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>348</v>
+        <v>411</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>349</v>
+        <v>412</v>
       </c>
       <c r="B20" s="1" t="n">
         <f aca="false">ROUND(Consolidated!N6+Consolidated!N7+Consolidated!N8-LV!N51,2)</f>
@@ -11808,47 +13863,47 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>350</v>
+        <v>413</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>351</v>
+        <v>414</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>352</v>
+        <v>415</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>353</v>
+        <v>416</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>354</v>
+        <v>417</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>355</v>
+        <v>418</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>356</v>
+        <v>419</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>357</v>
+        <v>420</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>358</v>
+        <v>421</v>
       </c>
       <c r="B30" s="1" t="n">
         <f aca="false">ROUND(Consolidated!N26-B9,0)</f>
@@ -11857,7 +13912,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>359</v>
+        <v>422</v>
       </c>
       <c r="B31" s="1" t="n">
         <f aca="false">ROUND(Consolidated!N23-B5,0)</f>
@@ -11866,10 +13921,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>360</v>
+        <v>423</v>
       </c>
       <c r="B32" s="1" t="n">
-        <f aca="false">ROUND(Consolidated!M38-(1461134-115),0)</f>
+        <f aca="false">ROUND(Consolidated!M38-(1451690.4510566-115),0)</f>
         <v>-0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Board portal: staffing note - needs counted from job start, no lead time
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EkVDtrr64Hp1gx17meyeHf
</commit_message>
<xml_diff>
--- a/models/SixPeak_OperatingBudget_2026-10-28.xlsx
+++ b/models/SixPeak_OperatingBudget_2026-10-28.xlsx
@@ -830,7 +830,7 @@
     <t xml:space="preserve">LV staffing: active jobs and people by role, April 2026 to December 2027</t>
   </si>
   <si>
-    <t xml:space="preserve">Requested by Chris Andresen (29 Oct 2026) to explain the FY2027 hires, the main expense item. Source: Base Case staffing engine and Personnel tab (models _2026-10-28). April 2026 is the first month of the model roster; payroll staffing schedules before June list only part of the team, so earlier months are not shown. "Needed" is the engine's requirement from the active jobs, including superintendent lead time before a start; a role is hired only when the need exceeds staff by 0.75 of a person, and PMs and APMs overlap a job's last 5 months.</t>
+    <t xml:space="preserve">Requested by Chris Andresen (29 Oct 2026) to explain the FY2027 hires, the main expense item. Source: Base Case staffing engine and Personnel tab (models _2026-10-28). April 2026 is the first month of the model roster; payroll staffing schedules before June list only part of the team, so earlier months are not shown. "Needed" is the engine's requirement from the active jobs, counted from each job's start month to one month after it finishes (no lead time before a start); a role is hired only when the need exceeds staff by 0.75 of a person, and PMs and APMs overlap a job's last 5 months.</t>
   </si>
   <si>
     <t xml:space="preserve">Month</t>
@@ -1528,7 +1528,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="61">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1705,79 +1705,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1795,14 +1771,6 @@
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -9104,46 +9072,46 @@
   <dimension ref="A1:V47"/>
   <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="5" style="0" width="8.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="5" style="1" width="8.5"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="44" t="s">
         <v>267</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
-      <c r="P2" s="45"/>
-      <c r="Q2" s="45"/>
-      <c r="R2" s="45"/>
-      <c r="S2" s="45"/>
-      <c r="T2" s="45"/>
-      <c r="U2" s="45"/>
-      <c r="V2" s="45"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="46" t="s">
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44"/>
+      <c r="S2" s="44"/>
+      <c r="T2" s="44"/>
+      <c r="U2" s="44"/>
+      <c r="V2" s="44"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>268</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -9210,1501 +9178,1501 @@
         <v>289</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="47" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
         <v>290</v>
       </c>
-      <c r="B5" s="48" t="n">
+      <c r="B5" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="48" t="n">
+      <c r="C5" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="D5" s="48" t="n">
+      <c r="D5" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="48" t="n">
+      <c r="E5" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="48" t="n">
+      <c r="F5" s="31" t="n">
         <v>7</v>
       </c>
-      <c r="G5" s="48" t="n">
+      <c r="G5" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="H5" s="48" t="n">
+      <c r="H5" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="I5" s="48" t="n">
+      <c r="I5" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="48" t="n">
+      <c r="J5" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="K5" s="48" t="n">
+      <c r="K5" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="L5" s="48" t="n">
+      <c r="L5" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="M5" s="48" t="n">
+      <c r="M5" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="N5" s="48" t="n">
+      <c r="N5" s="31" t="n">
         <v>11</v>
       </c>
-      <c r="O5" s="48" t="n">
+      <c r="O5" s="31" t="n">
         <v>12</v>
       </c>
-      <c r="P5" s="48" t="n">
+      <c r="P5" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="Q5" s="48" t="n">
+      <c r="Q5" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="R5" s="48" t="n">
+      <c r="R5" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="S5" s="48" t="n">
+      <c r="S5" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="T5" s="48" t="n">
+      <c r="T5" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="U5" s="48" t="n">
+      <c r="U5" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="V5" s="48" t="n">
+      <c r="V5" s="31" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="49" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="45" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="50" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
         <v>292</v>
       </c>
-      <c r="B8" s="51" t="n">
+      <c r="B8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="51" t="n">
+      <c r="D8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="51" t="n">
+      <c r="E8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="51" t="n">
+      <c r="F8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="51" t="n">
+      <c r="G8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="51" t="n">
+      <c r="H8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="I8" s="51" t="n">
+      <c r="I8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="J8" s="51" t="n">
+      <c r="J8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="K8" s="51" t="n">
+      <c r="K8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="L8" s="51" t="n">
+      <c r="L8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="M8" s="51" t="n">
+      <c r="M8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="N8" s="51" t="n">
+      <c r="N8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="O8" s="51" t="n">
+      <c r="O8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="P8" s="51" t="n">
+      <c r="P8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="Q8" s="51" t="n">
+      <c r="Q8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="R8" s="51" t="n">
+      <c r="R8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="S8" s="51" t="n">
+      <c r="S8" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="T8" s="51" t="n">
+      <c r="T8" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="U8" s="51" t="n">
+      <c r="U8" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="V8" s="51" t="n">
+      <c r="V8" s="46" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="52" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="47" t="s">
         <v>293</v>
       </c>
-      <c r="B9" s="53" t="n">
+      <c r="B9" s="48" t="n">
         <v>1.6</v>
       </c>
-      <c r="C9" s="53" t="n">
+      <c r="C9" s="48" t="n">
         <v>1.6</v>
       </c>
-      <c r="D9" s="53" t="n">
+      <c r="D9" s="48" t="n">
         <v>1.6</v>
       </c>
-      <c r="E9" s="53" t="n">
+      <c r="E9" s="48" t="n">
         <v>1.4</v>
       </c>
-      <c r="F9" s="53" t="n">
+      <c r="F9" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="53" t="n">
+      <c r="G9" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="H9" s="53" t="n">
+      <c r="H9" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="I9" s="53" t="n">
+      <c r="I9" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="J9" s="53" t="n">
+      <c r="J9" s="48" t="n">
         <v>2.5</v>
       </c>
-      <c r="K9" s="53" t="n">
+      <c r="K9" s="48" t="n">
         <v>2.7</v>
       </c>
-      <c r="L9" s="53" t="n">
+      <c r="L9" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="M9" s="53" t="n">
+      <c r="M9" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="N9" s="53" t="n">
+      <c r="N9" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="O9" s="53" t="n">
+      <c r="O9" s="48" t="n">
         <v>3.1</v>
       </c>
-      <c r="P9" s="53" t="n">
+      <c r="P9" s="48" t="n">
         <v>3.8</v>
       </c>
-      <c r="Q9" s="53" t="n">
+      <c r="Q9" s="48" t="n">
         <v>3.8</v>
       </c>
-      <c r="R9" s="53" t="n">
+      <c r="R9" s="48" t="n">
         <v>3.5</v>
       </c>
-      <c r="S9" s="53" t="n">
+      <c r="S9" s="48" t="n">
         <v>3.7</v>
       </c>
-      <c r="T9" s="53" t="n">
+      <c r="T9" s="48" t="n">
         <v>4.2</v>
       </c>
-      <c r="U9" s="53" t="n">
+      <c r="U9" s="48" t="n">
         <v>4</v>
       </c>
-      <c r="V9" s="53" t="n">
+      <c r="V9" s="48" t="n">
         <v>3.9</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="50" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
         <v>294</v>
       </c>
-      <c r="B10" s="51" t="n">
+      <c r="B10" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="51" t="n">
+      <c r="C10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="51" t="n">
+      <c r="D10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="51" t="n">
+      <c r="E10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="51" t="n">
+      <c r="F10" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="51" t="n">
+      <c r="G10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="51" t="n">
+      <c r="H10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="51" t="n">
+      <c r="I10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="J10" s="51" t="n">
+      <c r="J10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="K10" s="51" t="n">
+      <c r="K10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="L10" s="51" t="n">
+      <c r="L10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="M10" s="51" t="n">
+      <c r="M10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="N10" s="51" t="n">
+      <c r="N10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="O10" s="51" t="n">
+      <c r="O10" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="P10" s="51" t="n">
+      <c r="P10" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="Q10" s="51" t="n">
+      <c r="Q10" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="R10" s="51" t="n">
+      <c r="R10" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="S10" s="51" t="n">
+      <c r="S10" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="T10" s="51" t="n">
+      <c r="T10" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="U10" s="51" t="n">
+      <c r="U10" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="V10" s="51" t="n">
+      <c r="V10" s="46" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="52" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="47" t="s">
         <v>293</v>
       </c>
-      <c r="B11" s="53" t="n">
+      <c r="B11" s="48" t="n">
         <v>1.1</v>
       </c>
-      <c r="C11" s="53" t="n">
+      <c r="C11" s="48" t="n">
         <v>1.1</v>
       </c>
-      <c r="D11" s="53" t="n">
+      <c r="D11" s="48" t="n">
         <v>1.1</v>
       </c>
-      <c r="E11" s="53" t="n">
+      <c r="E11" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="53" t="n">
+      <c r="F11" s="48" t="n">
         <v>1.7</v>
       </c>
-      <c r="G11" s="53" t="n">
+      <c r="G11" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="53" t="n">
+      <c r="H11" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="I11" s="53" t="n">
+      <c r="I11" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="J11" s="53" t="n">
+      <c r="J11" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="K11" s="53" t="n">
+      <c r="K11" s="48" t="n">
         <v>2.3</v>
       </c>
-      <c r="L11" s="53" t="n">
+      <c r="L11" s="48" t="n">
         <v>2.4</v>
       </c>
-      <c r="M11" s="53" t="n">
+      <c r="M11" s="48" t="n">
         <v>2.4</v>
       </c>
-      <c r="N11" s="53" t="n">
+      <c r="N11" s="48" t="n">
         <v>2.5</v>
       </c>
-      <c r="O11" s="53" t="n">
+      <c r="O11" s="48" t="n">
         <v>2.7</v>
       </c>
-      <c r="P11" s="53" t="n">
+      <c r="P11" s="48" t="n">
         <v>3.3</v>
       </c>
-      <c r="Q11" s="53" t="n">
+      <c r="Q11" s="48" t="n">
         <v>3.3</v>
       </c>
-      <c r="R11" s="53" t="n">
+      <c r="R11" s="48" t="n">
         <v>3.2</v>
       </c>
-      <c r="S11" s="53" t="n">
+      <c r="S11" s="48" t="n">
         <v>3.5</v>
       </c>
-      <c r="T11" s="53" t="n">
+      <c r="T11" s="48" t="n">
         <v>4</v>
       </c>
-      <c r="U11" s="53" t="n">
+      <c r="U11" s="48" t="n">
         <v>3.7</v>
       </c>
-      <c r="V11" s="53" t="n">
+      <c r="V11" s="48" t="n">
         <v>3.6</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="50" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
         <v>295</v>
       </c>
-      <c r="B12" s="51" t="n">
+      <c r="B12" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="51" t="n">
+      <c r="C12" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="51" t="n">
+      <c r="D12" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="51" t="n">
+      <c r="E12" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="51" t="n">
+      <c r="F12" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="51" t="n">
+      <c r="G12" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="H12" s="51" t="n">
+      <c r="H12" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="I12" s="51" t="n">
+      <c r="I12" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="J12" s="51" t="n">
+      <c r="J12" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="K12" s="51" t="n">
+      <c r="K12" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="L12" s="51" t="n">
+      <c r="L12" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="M12" s="51" t="n">
+      <c r="M12" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="N12" s="51" t="n">
+      <c r="N12" s="46" t="n">
         <v>9</v>
       </c>
-      <c r="O12" s="51" t="n">
+      <c r="O12" s="46" t="n">
         <v>10</v>
       </c>
-      <c r="P12" s="51" t="n">
+      <c r="P12" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="Q12" s="51" t="n">
+      <c r="Q12" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="R12" s="51" t="n">
+      <c r="R12" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="S12" s="51" t="n">
+      <c r="S12" s="46" t="n">
         <v>12</v>
       </c>
-      <c r="T12" s="51" t="n">
+      <c r="T12" s="46" t="n">
         <v>13</v>
       </c>
-      <c r="U12" s="51" t="n">
+      <c r="U12" s="46" t="n">
         <v>13</v>
       </c>
-      <c r="V12" s="51" t="n">
+      <c r="V12" s="46" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="52" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="47" t="s">
         <v>293</v>
       </c>
-      <c r="B13" s="53" t="n">
+      <c r="B13" s="48" t="n">
         <v>4.4</v>
       </c>
-      <c r="C13" s="53" t="n">
+      <c r="C13" s="48" t="n">
         <v>4.4</v>
       </c>
-      <c r="D13" s="53" t="n">
+      <c r="D13" s="48" t="n">
         <v>4.4</v>
       </c>
-      <c r="E13" s="53" t="n">
+      <c r="E13" s="48" t="n">
         <v>4.4</v>
       </c>
-      <c r="F13" s="53" t="n">
+      <c r="F13" s="48" t="n">
         <v>6.1</v>
       </c>
-      <c r="G13" s="53" t="n">
+      <c r="G13" s="48" t="n">
         <v>7</v>
       </c>
-      <c r="H13" s="53" t="n">
+      <c r="H13" s="48" t="n">
         <v>7</v>
       </c>
-      <c r="I13" s="53" t="n">
+      <c r="I13" s="48" t="n">
         <v>7</v>
       </c>
-      <c r="J13" s="53" t="n">
+      <c r="J13" s="48" t="n">
         <v>7.9</v>
       </c>
-      <c r="K13" s="53" t="n">
+      <c r="K13" s="48" t="n">
         <v>7.9</v>
       </c>
-      <c r="L13" s="53" t="n">
+      <c r="L13" s="48" t="n">
         <v>8.8</v>
       </c>
-      <c r="M13" s="53" t="n">
+      <c r="M13" s="48" t="n">
         <v>8.8</v>
       </c>
-      <c r="N13" s="53" t="n">
+      <c r="N13" s="48" t="n">
         <v>9.6</v>
       </c>
-      <c r="O13" s="53" t="n">
+      <c r="O13" s="48" t="n">
         <v>10.5</v>
       </c>
-      <c r="P13" s="53" t="n">
+      <c r="P13" s="48" t="n">
         <v>12.2</v>
       </c>
-      <c r="Q13" s="53" t="n">
+      <c r="Q13" s="48" t="n">
         <v>12.2</v>
       </c>
-      <c r="R13" s="53" t="n">
+      <c r="R13" s="48" t="n">
         <v>11.4</v>
       </c>
-      <c r="S13" s="53" t="n">
+      <c r="S13" s="48" t="n">
         <v>12.2</v>
       </c>
-      <c r="T13" s="53" t="n">
+      <c r="T13" s="48" t="n">
         <v>13.1</v>
       </c>
-      <c r="U13" s="53" t="n">
+      <c r="U13" s="48" t="n">
         <v>12.2</v>
       </c>
-      <c r="V13" s="53" t="n">
+      <c r="V13" s="48" t="n">
         <v>11.4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="50" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
         <v>296</v>
       </c>
-      <c r="B14" s="51" t="n">
+      <c r="B14" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="51" t="n">
+      <c r="C14" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="51" t="n">
+      <c r="D14" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="51" t="n">
+      <c r="E14" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="51" t="n">
+      <c r="F14" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="G14" s="51" t="n">
+      <c r="G14" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="51" t="n">
+      <c r="H14" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="I14" s="51" t="n">
+      <c r="I14" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="J14" s="51" t="n">
+      <c r="J14" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="K14" s="51" t="n">
+      <c r="K14" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="L14" s="51" t="n">
+      <c r="L14" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="M14" s="51" t="n">
+      <c r="M14" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="N14" s="51" t="n">
+      <c r="N14" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="O14" s="51" t="n">
+      <c r="O14" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="P14" s="51" t="n">
+      <c r="P14" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="Q14" s="51" t="n">
+      <c r="Q14" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="R14" s="51" t="n">
+      <c r="R14" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="S14" s="51" t="n">
+      <c r="S14" s="46" t="n">
         <v>7</v>
       </c>
-      <c r="T14" s="51" t="n">
+      <c r="T14" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="U14" s="51" t="n">
+      <c r="U14" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="V14" s="51" t="n">
+      <c r="V14" s="46" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="52" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="47" t="s">
         <v>293</v>
       </c>
-      <c r="B15" s="53" t="n">
+      <c r="B15" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="C15" s="53" t="n">
+      <c r="C15" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="D15" s="53" t="n">
+      <c r="D15" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="E15" s="53" t="n">
+      <c r="E15" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="F15" s="53" t="n">
+      <c r="F15" s="48" t="n">
         <v>3.7</v>
       </c>
-      <c r="G15" s="53" t="n">
+      <c r="G15" s="48" t="n">
         <v>4.2</v>
       </c>
-      <c r="H15" s="53" t="n">
+      <c r="H15" s="48" t="n">
         <v>4.2</v>
       </c>
-      <c r="I15" s="53" t="n">
+      <c r="I15" s="48" t="n">
         <v>4.2</v>
       </c>
-      <c r="J15" s="53" t="n">
+      <c r="J15" s="48" t="n">
         <v>4.7</v>
       </c>
-      <c r="K15" s="53" t="n">
+      <c r="K15" s="48" t="n">
         <v>4.7</v>
       </c>
-      <c r="L15" s="53" t="n">
+      <c r="L15" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="M15" s="53" t="n">
+      <c r="M15" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="N15" s="53" t="n">
+      <c r="N15" s="48" t="n">
         <v>5.5</v>
       </c>
-      <c r="O15" s="53" t="n">
+      <c r="O15" s="48" t="n">
         <v>6</v>
       </c>
-      <c r="P15" s="53" t="n">
+      <c r="P15" s="48" t="n">
         <v>7.5</v>
       </c>
-      <c r="Q15" s="53" t="n">
+      <c r="Q15" s="48" t="n">
         <v>7.5</v>
       </c>
-      <c r="R15" s="53" t="n">
+      <c r="R15" s="48" t="n">
         <v>7.2</v>
       </c>
-      <c r="S15" s="53" t="n">
+      <c r="S15" s="48" t="n">
         <v>7.7</v>
       </c>
-      <c r="T15" s="53" t="n">
+      <c r="T15" s="48" t="n">
         <v>8.7</v>
       </c>
-      <c r="U15" s="53" t="n">
+      <c r="U15" s="48" t="n">
         <v>8.2</v>
       </c>
-      <c r="V15" s="53" t="n">
+      <c r="V15" s="48" t="n">
         <v>7.7</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="50" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
         <v>297</v>
       </c>
-      <c r="B16" s="51" t="n">
+      <c r="B16" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="51" t="n">
+      <c r="C16" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="51" t="n">
+      <c r="D16" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="51" t="n">
+      <c r="E16" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="51" t="n">
+      <c r="F16" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="51" t="n">
+      <c r="G16" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="51" t="n">
+      <c r="H16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="I16" s="51" t="n">
+      <c r="I16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="J16" s="51" t="n">
+      <c r="J16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="K16" s="51" t="n">
+      <c r="K16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="L16" s="51" t="n">
+      <c r="L16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="M16" s="51" t="n">
+      <c r="M16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="N16" s="51" t="n">
+      <c r="N16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="O16" s="51" t="n">
+      <c r="O16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="P16" s="51" t="n">
+      <c r="P16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="Q16" s="51" t="n">
+      <c r="Q16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="R16" s="51" t="n">
+      <c r="R16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="S16" s="51" t="n">
+      <c r="S16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="T16" s="51" t="n">
+      <c r="T16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="U16" s="51" t="n">
+      <c r="U16" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="V16" s="51" t="n">
+      <c r="V16" s="46" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="50" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
         <v>298</v>
       </c>
-      <c r="B17" s="51" t="n">
+      <c r="B17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="C17" s="51" t="n">
+      <c r="C17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="51" t="n">
+      <c r="D17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="E17" s="51" t="n">
+      <c r="E17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="51" t="n">
+      <c r="F17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="G17" s="51" t="n">
+      <c r="G17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="H17" s="51" t="n">
+      <c r="H17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="51" t="n">
+      <c r="I17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="J17" s="51" t="n">
+      <c r="J17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="K17" s="51" t="n">
+      <c r="K17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="L17" s="51" t="n">
+      <c r="L17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="M17" s="51" t="n">
+      <c r="M17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="N17" s="51" t="n">
+      <c r="N17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="O17" s="51" t="n">
+      <c r="O17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="P17" s="51" t="n">
+      <c r="P17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="Q17" s="51" t="n">
+      <c r="Q17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="R17" s="51" t="n">
+      <c r="R17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="S17" s="51" t="n">
+      <c r="S17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="T17" s="51" t="n">
+      <c r="T17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="U17" s="51" t="n">
+      <c r="U17" s="46" t="n">
         <v>4</v>
       </c>
-      <c r="V17" s="51" t="n">
+      <c r="V17" s="46" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="50" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
         <v>299</v>
       </c>
-      <c r="B18" s="51" t="n">
+      <c r="B18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="51" t="n">
+      <c r="C18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="D18" s="51" t="n">
+      <c r="D18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="51" t="n">
+      <c r="E18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="F18" s="51" t="n">
+      <c r="F18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="51" t="n">
+      <c r="G18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="H18" s="51" t="n">
+      <c r="H18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="51" t="n">
+      <c r="I18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="J18" s="51" t="n">
+      <c r="J18" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="K18" s="51" t="n">
+      <c r="K18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="L18" s="51" t="n">
+      <c r="L18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="M18" s="51" t="n">
+      <c r="M18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="N18" s="51" t="n">
+      <c r="N18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="O18" s="51" t="n">
+      <c r="O18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="P18" s="51" t="n">
+      <c r="P18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="Q18" s="51" t="n">
+      <c r="Q18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="R18" s="51" t="n">
+      <c r="R18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="S18" s="51" t="n">
+      <c r="S18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="T18" s="51" t="n">
+      <c r="T18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="U18" s="51" t="n">
+      <c r="U18" s="46" t="n">
         <v>2</v>
       </c>
-      <c r="V18" s="51" t="n">
+      <c r="V18" s="46" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="54" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="49" t="s">
         <v>300</v>
       </c>
-      <c r="B19" s="55" t="n">
+      <c r="B19" s="50" t="n">
         <f aca="false">B8+B10+B12+B14+B16+B17+B18</f>
         <v>17</v>
       </c>
-      <c r="C19" s="55" t="n">
+      <c r="C19" s="50" t="n">
         <f aca="false">C8+C10+C12+C14+C16+C17+C18</f>
         <v>19</v>
       </c>
-      <c r="D19" s="55" t="n">
+      <c r="D19" s="50" t="n">
         <f aca="false">D8+D10+D12+D14+D16+D17+D18</f>
         <v>22</v>
       </c>
-      <c r="E19" s="55" t="n">
+      <c r="E19" s="50" t="n">
         <f aca="false">E8+E10+E12+E14+E16+E17+E18</f>
         <v>23</v>
       </c>
-      <c r="F19" s="55" t="n">
+      <c r="F19" s="50" t="n">
         <f aca="false">F8+F10+F12+F14+F16+F17+F18</f>
         <v>23</v>
       </c>
-      <c r="G19" s="55" t="n">
+      <c r="G19" s="50" t="n">
         <f aca="false">G8+G10+G12+G14+G16+G17+G18</f>
         <v>25</v>
       </c>
-      <c r="H19" s="55" t="n">
+      <c r="H19" s="50" t="n">
         <f aca="false">H8+H10+H12+H14+H16+H17+H18</f>
         <v>26</v>
       </c>
-      <c r="I19" s="55" t="n">
+      <c r="I19" s="50" t="n">
         <f aca="false">I8+I10+I12+I14+I16+I17+I18</f>
         <v>26</v>
       </c>
-      <c r="J19" s="55" t="n">
+      <c r="J19" s="50" t="n">
         <f aca="false">J8+J10+J12+J14+J16+J17+J18</f>
         <v>27</v>
       </c>
-      <c r="K19" s="55" t="n">
+      <c r="K19" s="50" t="n">
         <f aca="false">K8+K10+K12+K14+K16+K17+K18</f>
         <v>26</v>
       </c>
-      <c r="L19" s="55" t="n">
+      <c r="L19" s="50" t="n">
         <f aca="false">L8+L10+L12+L14+L16+L17+L18</f>
         <v>27</v>
       </c>
-      <c r="M19" s="55" t="n">
+      <c r="M19" s="50" t="n">
         <f aca="false">M8+M10+M12+M14+M16+M17+M18</f>
         <v>27</v>
       </c>
-      <c r="N19" s="55" t="n">
+      <c r="N19" s="50" t="n">
         <f aca="false">N8+N10+N12+N14+N16+N17+N18</f>
         <v>28</v>
       </c>
-      <c r="O19" s="55" t="n">
+      <c r="O19" s="50" t="n">
         <f aca="false">O8+O10+O12+O14+O16+O17+O18</f>
         <v>30</v>
       </c>
-      <c r="P19" s="55" t="n">
+      <c r="P19" s="50" t="n">
         <f aca="false">P8+P10+P12+P14+P16+P17+P18</f>
         <v>34</v>
       </c>
-      <c r="Q19" s="55" t="n">
+      <c r="Q19" s="50" t="n">
         <f aca="false">Q8+Q10+Q12+Q14+Q16+Q17+Q18</f>
         <v>34</v>
       </c>
-      <c r="R19" s="55" t="n">
+      <c r="R19" s="50" t="n">
         <f aca="false">R8+R10+R12+R14+R16+R17+R18</f>
         <v>34</v>
       </c>
-      <c r="S19" s="55" t="n">
+      <c r="S19" s="50" t="n">
         <f aca="false">S8+S10+S12+S14+S16+S17+S18</f>
         <v>34</v>
       </c>
-      <c r="T19" s="55" t="n">
+      <c r="T19" s="50" t="n">
         <f aca="false">T8+T10+T12+T14+T16+T17+T18</f>
         <v>38</v>
       </c>
-      <c r="U19" s="55" t="n">
+      <c r="U19" s="50" t="n">
         <f aca="false">U8+U10+U12+U14+U16+U17+U18</f>
         <v>38</v>
       </c>
-      <c r="V19" s="55" t="n">
+      <c r="V19" s="50" t="n">
         <f aca="false">V8+V10+V12+V14+V16+V17+V18</f>
         <v>38</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="52" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="47" t="s">
         <v>301</v>
       </c>
-      <c r="B20" s="56"/>
-      <c r="C20" s="56" t="n">
+      <c r="B20" s="51"/>
+      <c r="C20" s="51" t="n">
         <f aca="false">C19-B19</f>
         <v>2</v>
       </c>
-      <c r="D20" s="56" t="n">
+      <c r="D20" s="51" t="n">
         <f aca="false">D19-C19</f>
         <v>3</v>
       </c>
-      <c r="E20" s="56" t="n">
+      <c r="E20" s="51" t="n">
         <f aca="false">E19-D19</f>
         <v>1</v>
       </c>
-      <c r="F20" s="56" t="n">
+      <c r="F20" s="51" t="n">
         <f aca="false">F19-E19</f>
         <v>0</v>
       </c>
-      <c r="G20" s="56" t="n">
+      <c r="G20" s="51" t="n">
         <f aca="false">G19-F19</f>
         <v>2</v>
       </c>
-      <c r="H20" s="56" t="n">
+      <c r="H20" s="51" t="n">
         <f aca="false">H19-G19</f>
         <v>1</v>
       </c>
-      <c r="I20" s="56" t="n">
+      <c r="I20" s="51" t="n">
         <f aca="false">I19-H19</f>
         <v>0</v>
       </c>
-      <c r="J20" s="56" t="n">
+      <c r="J20" s="51" t="n">
         <f aca="false">J19-I19</f>
         <v>1</v>
       </c>
-      <c r="K20" s="56" t="n">
+      <c r="K20" s="51" t="n">
         <f aca="false">K19-J19</f>
         <v>-1</v>
       </c>
-      <c r="L20" s="56" t="n">
+      <c r="L20" s="51" t="n">
         <f aca="false">L19-K19</f>
         <v>1</v>
       </c>
-      <c r="M20" s="56" t="n">
+      <c r="M20" s="51" t="n">
         <f aca="false">M19-L19</f>
         <v>0</v>
       </c>
-      <c r="N20" s="56" t="n">
+      <c r="N20" s="51" t="n">
         <f aca="false">N19-M19</f>
         <v>1</v>
       </c>
-      <c r="O20" s="56" t="n">
+      <c r="O20" s="51" t="n">
         <f aca="false">O19-N19</f>
         <v>2</v>
       </c>
-      <c r="P20" s="56" t="n">
+      <c r="P20" s="51" t="n">
         <f aca="false">P19-O19</f>
         <v>4</v>
       </c>
-      <c r="Q20" s="56" t="n">
+      <c r="Q20" s="51" t="n">
         <f aca="false">Q19-P19</f>
         <v>0</v>
       </c>
-      <c r="R20" s="56" t="n">
+      <c r="R20" s="51" t="n">
         <f aca="false">R19-Q19</f>
         <v>0</v>
       </c>
-      <c r="S20" s="56" t="n">
+      <c r="S20" s="51" t="n">
         <f aca="false">S19-R19</f>
         <v>0</v>
       </c>
-      <c r="T20" s="56" t="n">
+      <c r="T20" s="51" t="n">
         <f aca="false">T19-S19</f>
         <v>4</v>
       </c>
-      <c r="U20" s="56" t="n">
+      <c r="U20" s="51" t="n">
         <f aca="false">U19-T19</f>
         <v>0</v>
       </c>
-      <c r="V20" s="56" t="n">
+      <c r="V20" s="51" t="n">
         <f aca="false">V19-U19</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
         <v>302</v>
       </c>
-      <c r="B22" s="51" t="n">
+      <c r="B22" s="46" t="n">
         <v>187694</v>
       </c>
-      <c r="C22" s="51" t="n">
+      <c r="C22" s="46" t="n">
         <v>295949</v>
       </c>
-      <c r="D22" s="51" t="n">
+      <c r="D22" s="46" t="n">
         <v>198646</v>
       </c>
-      <c r="E22" s="51" t="n">
+      <c r="E22" s="46" t="n">
         <v>215852</v>
       </c>
-      <c r="F22" s="51" t="n">
+      <c r="F22" s="46" t="n">
         <v>217611</v>
       </c>
-      <c r="G22" s="51" t="n">
+      <c r="G22" s="46" t="n">
         <v>223657</v>
       </c>
-      <c r="H22" s="51" t="n">
+      <c r="H22" s="46" t="n">
         <v>267964</v>
       </c>
-      <c r="I22" s="51" t="n">
+      <c r="I22" s="46" t="n">
         <v>267964</v>
       </c>
-      <c r="J22" s="51" t="n">
+      <c r="J22" s="46" t="n">
         <v>356298</v>
       </c>
-      <c r="K22" s="51" t="n">
+      <c r="K22" s="46" t="n">
         <v>270881</v>
       </c>
-      <c r="L22" s="51" t="n">
+      <c r="L22" s="46" t="n">
         <v>281298</v>
       </c>
-      <c r="M22" s="51" t="n">
+      <c r="M22" s="46" t="n">
         <v>281298</v>
       </c>
-      <c r="N22" s="51" t="n">
+      <c r="N22" s="46" t="n">
         <v>294631</v>
       </c>
-      <c r="O22" s="51" t="n">
+      <c r="O22" s="46" t="n">
         <v>318381</v>
       </c>
-      <c r="P22" s="51" t="n">
+      <c r="P22" s="46" t="n">
         <v>366298</v>
       </c>
-      <c r="Q22" s="51" t="n">
+      <c r="Q22" s="46" t="n">
         <v>366298</v>
       </c>
-      <c r="R22" s="51" t="n">
+      <c r="R22" s="46" t="n">
         <v>366298</v>
       </c>
-      <c r="S22" s="51" t="n">
+      <c r="S22" s="46" t="n">
         <v>366298</v>
       </c>
-      <c r="T22" s="51" t="n">
+      <c r="T22" s="46" t="n">
         <v>415881</v>
       </c>
-      <c r="U22" s="51" t="n">
+      <c r="U22" s="46" t="n">
         <v>415881</v>
       </c>
-      <c r="V22" s="51" t="n">
+      <c r="V22" s="46" t="n">
         <v>615881</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="57" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="B23" s="58" t="n">
+      <c r="B23" s="52" t="n">
         <f aca="false">B22/B5</f>
         <v>37538.8</v>
       </c>
-      <c r="C23" s="58" t="n">
+      <c r="C23" s="52" t="n">
         <f aca="false">C22/C5</f>
         <v>59189.8</v>
       </c>
-      <c r="D23" s="58" t="n">
+      <c r="D23" s="52" t="n">
         <f aca="false">D22/D5</f>
         <v>39729.2</v>
       </c>
-      <c r="E23" s="58" t="n">
+      <c r="E23" s="52" t="n">
         <f aca="false">E22/E5</f>
         <v>43170.4</v>
       </c>
-      <c r="F23" s="58" t="n">
+      <c r="F23" s="52" t="n">
         <f aca="false">F22/F5</f>
         <v>31087.2857142857</v>
       </c>
-      <c r="G23" s="58" t="n">
+      <c r="G23" s="52" t="n">
         <f aca="false">G22/G5</f>
         <v>27957.125</v>
       </c>
-      <c r="H23" s="58" t="n">
+      <c r="H23" s="52" t="n">
         <f aca="false">H22/H5</f>
         <v>33495.5</v>
       </c>
-      <c r="I23" s="58" t="n">
+      <c r="I23" s="52" t="n">
         <f aca="false">I22/I5</f>
         <v>33495.5</v>
       </c>
-      <c r="J23" s="58" t="n">
+      <c r="J23" s="52" t="n">
         <f aca="false">J22/J5</f>
         <v>44537.25</v>
       </c>
-      <c r="K23" s="58" t="n">
+      <c r="K23" s="52" t="n">
         <f aca="false">K22/K5</f>
         <v>30097.8888888889</v>
       </c>
-      <c r="L23" s="58" t="n">
+      <c r="L23" s="52" t="n">
         <f aca="false">L22/L5</f>
         <v>28129.8</v>
       </c>
-      <c r="M23" s="58" t="n">
+      <c r="M23" s="52" t="n">
         <f aca="false">M22/M5</f>
         <v>28129.8</v>
       </c>
-      <c r="N23" s="58" t="n">
+      <c r="N23" s="52" t="n">
         <f aca="false">N22/N5</f>
         <v>26784.6363636364</v>
       </c>
-      <c r="O23" s="58" t="n">
+      <c r="O23" s="52" t="n">
         <f aca="false">O22/O5</f>
         <v>26531.75</v>
       </c>
-      <c r="P23" s="58" t="n">
+      <c r="P23" s="52" t="n">
         <f aca="false">P22/P5</f>
         <v>26164.1428571429</v>
       </c>
-      <c r="Q23" s="58" t="n">
+      <c r="Q23" s="52" t="n">
         <f aca="false">Q22/Q5</f>
         <v>28176.7692307692</v>
       </c>
-      <c r="R23" s="58" t="n">
+      <c r="R23" s="52" t="n">
         <f aca="false">R22/R5</f>
         <v>28176.7692307692</v>
       </c>
-      <c r="S23" s="58" t="n">
+      <c r="S23" s="52" t="n">
         <f aca="false">S22/S5</f>
         <v>28176.7692307692</v>
       </c>
-      <c r="T23" s="58" t="n">
+      <c r="T23" s="52" t="n">
         <f aca="false">T22/T5</f>
         <v>29705.7857142857</v>
       </c>
-      <c r="U23" s="58" t="n">
+      <c r="U23" s="52" t="n">
         <f aca="false">U22/U5</f>
         <v>31990.8461538462</v>
       </c>
-      <c r="V23" s="58" t="n">
+      <c r="V23" s="52" t="n">
         <f aca="false">V22/V5</f>
         <v>47375.4615384615</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="57" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B24" s="59" t="n">
+      <c r="B24" s="53" t="n">
         <f aca="false">B5/B8</f>
         <v>1.66666666666667</v>
       </c>
-      <c r="C24" s="59" t="n">
+      <c r="C24" s="53" t="n">
         <f aca="false">C5/C8</f>
         <v>1.66666666666667</v>
       </c>
-      <c r="D24" s="59" t="n">
+      <c r="D24" s="53" t="n">
         <f aca="false">D5/D8</f>
         <v>1.66666666666667</v>
       </c>
-      <c r="E24" s="59" t="n">
+      <c r="E24" s="53" t="n">
         <f aca="false">E5/E8</f>
         <v>1.66666666666667</v>
       </c>
-      <c r="F24" s="59" t="n">
+      <c r="F24" s="53" t="n">
         <f aca="false">F5/F8</f>
         <v>2.33333333333333</v>
       </c>
-      <c r="G24" s="59" t="n">
+      <c r="G24" s="53" t="n">
         <f aca="false">G5/G8</f>
         <v>2.66666666666667</v>
       </c>
-      <c r="H24" s="59" t="n">
+      <c r="H24" s="53" t="n">
         <f aca="false">H5/H8</f>
         <v>2.66666666666667</v>
       </c>
-      <c r="I24" s="59" t="n">
+      <c r="I24" s="53" t="n">
         <f aca="false">I5/I8</f>
         <v>2.66666666666667</v>
       </c>
-      <c r="J24" s="59" t="n">
+      <c r="J24" s="53" t="n">
         <f aca="false">J5/J8</f>
         <v>2.66666666666667</v>
       </c>
-      <c r="K24" s="59" t="n">
+      <c r="K24" s="53" t="n">
         <f aca="false">K5/K8</f>
         <v>3</v>
       </c>
-      <c r="L24" s="59" t="n">
+      <c r="L24" s="53" t="n">
         <f aca="false">L5/L8</f>
         <v>3.33333333333333</v>
       </c>
-      <c r="M24" s="59" t="n">
+      <c r="M24" s="53" t="n">
         <f aca="false">M5/M8</f>
         <v>3.33333333333333</v>
       </c>
-      <c r="N24" s="59" t="n">
+      <c r="N24" s="53" t="n">
         <f aca="false">N5/N8</f>
         <v>3.66666666666667</v>
       </c>
-      <c r="O24" s="59" t="n">
+      <c r="O24" s="53" t="n">
         <f aca="false">O5/O8</f>
         <v>4</v>
       </c>
-      <c r="P24" s="59" t="n">
+      <c r="P24" s="53" t="n">
         <f aca="false">P5/P8</f>
         <v>4.66666666666667</v>
       </c>
-      <c r="Q24" s="59" t="n">
+      <c r="Q24" s="53" t="n">
         <f aca="false">Q5/Q8</f>
         <v>4.33333333333333</v>
       </c>
-      <c r="R24" s="59" t="n">
+      <c r="R24" s="53" t="n">
         <f aca="false">R5/R8</f>
         <v>4.33333333333333</v>
       </c>
-      <c r="S24" s="59" t="n">
+      <c r="S24" s="53" t="n">
         <f aca="false">S5/S8</f>
         <v>4.33333333333333</v>
       </c>
-      <c r="T24" s="59" t="n">
+      <c r="T24" s="53" t="n">
         <f aca="false">T5/T8</f>
         <v>3.5</v>
       </c>
-      <c r="U24" s="59" t="n">
+      <c r="U24" s="53" t="n">
         <f aca="false">U5/U8</f>
         <v>3.25</v>
       </c>
-      <c r="V24" s="59" t="n">
+      <c r="V24" s="53" t="n">
         <f aca="false">V5/V8</f>
         <v>3.25</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="60" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="54" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="46" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
         <v>306</v>
       </c>
-      <c r="B27" s="46" t="s">
+      <c r="B27" s="4" t="s">
         <v>307</v>
       </c>
-      <c r="C27" s="46" t="s">
+      <c r="C27" s="4" t="s">
         <v>308</v>
       </c>
-      <c r="D27" s="46" t="s">
+      <c r="D27" s="4" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="57" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="B28" s="59" t="n">
+      <c r="B28" s="53" t="n">
         <f aca="false">AVERAGE(B5:J5)</f>
         <v>6.55555555555556</v>
       </c>
-      <c r="C28" s="59" t="n">
+      <c r="C28" s="53" t="n">
         <f aca="false">AVERAGE(K5:V5)</f>
         <v>12.0833333333333</v>
       </c>
-      <c r="D28" s="59" t="n">
+      <c r="D28" s="53" t="n">
         <f aca="false">C28-B28</f>
         <v>5.52777777777778</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="57" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="B29" s="58" t="n">
+      <c r="B29" s="52" t="n">
         <f aca="false">J5</f>
         <v>8</v>
       </c>
-      <c r="C29" s="58" t="n">
+      <c r="C29" s="52" t="n">
         <f aca="false">V5</f>
         <v>13</v>
       </c>
-      <c r="D29" s="58" t="n">
+      <c r="D29" s="52" t="n">
         <f aca="false">C29-B29</f>
         <v>5</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="57" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B30" s="59" t="n">
+      <c r="B30" s="53" t="n">
         <f aca="false">AVERAGE(B19:J19)</f>
         <v>23.1111111111111</v>
       </c>
-      <c r="C30" s="59" t="n">
+      <c r="C30" s="53" t="n">
         <f aca="false">AVERAGE(K19:V19)</f>
         <v>32.3333333333333</v>
       </c>
-      <c r="D30" s="59" t="n">
+      <c r="D30" s="53" t="n">
         <f aca="false">C30-B30</f>
         <v>9.22222222222223</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="57" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="B31" s="58" t="n">
+      <c r="B31" s="52" t="n">
         <f aca="false">J19</f>
         <v>27</v>
       </c>
-      <c r="C31" s="58" t="n">
+      <c r="C31" s="52" t="n">
         <f aca="false">V19</f>
         <v>38</v>
       </c>
-      <c r="D31" s="58" t="n">
+      <c r="D31" s="52" t="n">
         <f aca="false">C31-B31</f>
         <v>11</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="57" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B32" s="58" t="n">
+      <c r="B32" s="52" t="n">
         <f aca="false">J8</f>
         <v>3</v>
       </c>
-      <c r="C32" s="58" t="n">
+      <c r="C32" s="52" t="n">
         <f aca="false">V8</f>
         <v>4</v>
       </c>
-      <c r="D32" s="58" t="n">
+      <c r="D32" s="52" t="n">
         <f aca="false">C32-B32</f>
         <v>1</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="57" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B33" s="58" t="n">
+      <c r="B33" s="52" t="n">
         <f aca="false">J10</f>
         <v>2</v>
       </c>
-      <c r="C33" s="58" t="n">
+      <c r="C33" s="52" t="n">
         <f aca="false">V10</f>
         <v>4</v>
       </c>
-      <c r="D33" s="58" t="n">
+      <c r="D33" s="52" t="n">
         <f aca="false">C33-B33</f>
         <v>2</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="57" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="B34" s="58" t="n">
+      <c r="B34" s="52" t="n">
         <f aca="false">J12</f>
         <v>8</v>
       </c>
-      <c r="C34" s="58" t="n">
+      <c r="C34" s="52" t="n">
         <f aca="false">V12</f>
         <v>13</v>
       </c>
-      <c r="D34" s="58" t="n">
+      <c r="D34" s="52" t="n">
         <f aca="false">C34-B34</f>
         <v>5</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="57" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="B35" s="58" t="n">
+      <c r="B35" s="52" t="n">
         <f aca="false">J14</f>
         <v>4</v>
       </c>
-      <c r="C35" s="58" t="n">
+      <c r="C35" s="52" t="n">
         <f aca="false">V14</f>
         <v>8</v>
       </c>
-      <c r="D35" s="58" t="n">
+      <c r="D35" s="52" t="n">
         <f aca="false">C35-B35</f>
         <v>4</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="57" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="B36" s="58" t="n">
+      <c r="B36" s="52" t="n">
         <f aca="false">J16</f>
         <v>3</v>
       </c>
-      <c r="C36" s="58" t="n">
+      <c r="C36" s="52" t="n">
         <f aca="false">V16</f>
         <v>3</v>
       </c>
-      <c r="D36" s="58" t="n">
+      <c r="D36" s="52" t="n">
         <f aca="false">C36-B36</f>
         <v>0</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="57" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="B37" s="58" t="n">
+      <c r="B37" s="52" t="n">
         <f aca="false">J17</f>
         <v>4</v>
       </c>
-      <c r="C37" s="58" t="n">
+      <c r="C37" s="52" t="n">
         <f aca="false">V17</f>
         <v>4</v>
       </c>
-      <c r="D37" s="58" t="n">
+      <c r="D37" s="52" t="n">
         <f aca="false">C37-B37</f>
         <v>0</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="57" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B38" s="58" t="n">
+      <c r="B38" s="52" t="n">
         <f aca="false">J18</f>
         <v>3</v>
       </c>
-      <c r="C38" s="58" t="n">
+      <c r="C38" s="52" t="n">
         <f aca="false">V18</f>
         <v>2</v>
       </c>
-      <c r="D38" s="58" t="n">
+      <c r="D38" s="52" t="n">
         <f aca="false">C38-B38</f>
         <v>-1</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="57" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="B39" s="61" t="n">
+      <c r="B39" s="55" t="n">
         <f aca="false">AVERAGE(B5:J5)/AVERAGE(B8:J8)</f>
         <v>2.18518518518519</v>
       </c>
-      <c r="C39" s="61" t="n">
+      <c r="C39" s="55" t="n">
         <f aca="false">AVERAGE(K5:V5)/AVERAGE(K8:V8)</f>
         <v>3.71794871794872</v>
       </c>
-      <c r="D39" s="61" t="n">
+      <c r="D39" s="55" t="n">
         <f aca="false">C39-B39</f>
         <v>1.53276353276353</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="57" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B40" s="62" t="n">
+      <c r="B40" s="56" t="n">
         <f aca="false">AVERAGE(B5:J5)/AVERAGE(B12:J12)</f>
         <v>1.07272727272727</v>
       </c>
-      <c r="C40" s="62" t="n">
+      <c r="C40" s="56" t="n">
         <f aca="false">AVERAGE(K5:V5)/AVERAGE(K12:V12)</f>
         <v>1.11538461538462</v>
       </c>
-      <c r="D40" s="62" t="n">
+      <c r="D40" s="56" t="n">
         <f aca="false">C40-B40</f>
         <v>0.0426573426573427</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="57" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="B41" s="58" t="n">
+      <c r="B41" s="52" t="n">
         <f aca="false">SUM(B22:J22)/SUM(B5:J5)</f>
         <v>37824.3220338983</v>
       </c>
-      <c r="C41" s="58" t="n">
+      <c r="C41" s="52" t="n">
         <f aca="false">SUM(K22:V22)/SUM(K5:V5)</f>
         <v>30064.3034482759</v>
       </c>
-      <c r="D41" s="58" t="n">
+      <c r="D41" s="52" t="n">
         <f aca="false">C41-B41</f>
         <v>-7760.01858562245</v>
       </c>
@@ -13210,7 +13178,7 @@
       <c r="K20" s="36"/>
       <c r="L20" s="36"/>
       <c r="M20" s="36"/>
-      <c r="N20" s="63" t="n">
+      <c r="N20" s="57" t="n">
         <v>172240.34</v>
       </c>
     </row>
@@ -13230,7 +13198,7 @@
       <c r="K21" s="36"/>
       <c r="L21" s="36"/>
       <c r="M21" s="36"/>
-      <c r="N21" s="63" t="n">
+      <c r="N21" s="57" t="n">
         <v>25000</v>
       </c>
     </row>
@@ -13250,7 +13218,7 @@
       <c r="K22" s="36"/>
       <c r="L22" s="36"/>
       <c r="M22" s="36"/>
-      <c r="N22" s="63" t="n">
+      <c r="N22" s="57" t="n">
         <v>150000</v>
       </c>
     </row>
@@ -13270,7 +13238,7 @@
       <c r="K23" s="36"/>
       <c r="L23" s="36"/>
       <c r="M23" s="36"/>
-      <c r="N23" s="63" t="n">
+      <c r="N23" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13290,7 +13258,7 @@
       <c r="K24" s="36"/>
       <c r="L24" s="36"/>
       <c r="M24" s="36"/>
-      <c r="N24" s="63" t="n">
+      <c r="N24" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13310,7 +13278,7 @@
       <c r="K25" s="36"/>
       <c r="L25" s="36"/>
       <c r="M25" s="36"/>
-      <c r="N25" s="63" t="n">
+      <c r="N25" s="57" t="n">
         <v>800</v>
       </c>
     </row>
@@ -13330,7 +13298,7 @@
       <c r="K26" s="36"/>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
-      <c r="N26" s="63" t="n">
+      <c r="N26" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13350,7 +13318,7 @@
       <c r="K27" s="36"/>
       <c r="L27" s="36"/>
       <c r="M27" s="36"/>
-      <c r="N27" s="63" t="n">
+      <c r="N27" s="57" t="n">
         <v>-3559.66000000002</v>
       </c>
     </row>
@@ -13370,7 +13338,7 @@
       <c r="K28" s="36"/>
       <c r="L28" s="36"/>
       <c r="M28" s="36"/>
-      <c r="N28" s="63" t="n">
+      <c r="N28" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13390,7 +13358,7 @@
       <c r="K29" s="36"/>
       <c r="L29" s="36"/>
       <c r="M29" s="36"/>
-      <c r="N29" s="63" t="n">
+      <c r="N29" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13410,7 +13378,7 @@
       <c r="K30" s="36"/>
       <c r="L30" s="36"/>
       <c r="M30" s="36"/>
-      <c r="N30" s="63" t="n">
+      <c r="N30" s="57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13430,7 +13398,7 @@
       <c r="K31" s="36"/>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
-      <c r="N31" s="63" t="n">
+      <c r="N31" s="57" t="n">
         <v>3559.66000000002</v>
       </c>
     </row>
@@ -13450,7 +13418,7 @@
       <c r="K32" s="36"/>
       <c r="L32" s="36"/>
       <c r="M32" s="36"/>
-      <c r="N32" s="63" t="n">
+      <c r="N32" s="57" t="n">
         <v>3559.66000000003</v>
       </c>
     </row>
@@ -13483,12 +13451,12 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="58" t="s">
         <v>375</v>
       </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
@@ -13512,7 +13480,7 @@
         <f aca="false">-'Six Peak'!N29*222000/337000</f>
         <v>222000</v>
       </c>
-      <c r="C5" s="65" t="n">
+      <c r="C5" s="59" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="9" t="n">
@@ -13528,7 +13496,7 @@
         <f aca="false">-(('Six Peak'!N13+'Six Peak'!N14+'Six Peak'!N16+'Six Peak'!N17)*157500/657500+'Six Peak'!N15/3)</f>
         <v>221014.5</v>
       </c>
-      <c r="C6" s="65" t="n">
+      <c r="C6" s="59" t="n">
         <v>0.9</v>
       </c>
       <c r="D6" s="9" t="n">
@@ -13544,7 +13512,7 @@
         <f aca="false">-(('Six Peak'!N13+'Six Peak'!N14+'Six Peak'!N16+'Six Peak'!N17)*250000/657500+'Six Peak'!N15/3)</f>
         <v>322302</v>
       </c>
-      <c r="C7" s="65" t="n">
+      <c r="C7" s="59" t="n">
         <v>0.75</v>
       </c>
       <c r="D7" s="9" t="n">
@@ -13560,7 +13528,7 @@
         <f aca="false">-'Six Peak'!N34/2</f>
         <v>400000</v>
       </c>
-      <c r="C8" s="65" t="n">
+      <c r="C8" s="59" t="n">
         <v>0.5</v>
       </c>
       <c r="D8" s="9" t="n">
@@ -13576,7 +13544,7 @@
         <f aca="false">-'Six Peak'!N34/2</f>
         <v>400000</v>
       </c>
-      <c r="C9" s="65" t="n">
+      <c r="C9" s="59" t="n">
         <v>0.1</v>
       </c>
       <c r="D9" s="9" t="n">
@@ -13592,7 +13560,7 @@
         <f aca="false">-(('Six Peak'!N13+'Six Peak'!N14+'Six Peak'!N16+'Six Peak'!N17)*250000/657500+'Six Peak'!N15/3)</f>
         <v>322302</v>
       </c>
-      <c r="C10" s="65" t="n">
+      <c r="C10" s="59" t="n">
         <v>0.1</v>
       </c>
       <c r="D10" s="9" t="n">
@@ -13615,12 +13583,12 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="66" t="s">
+      <c r="A12" s="60" t="s">
         <v>386</v>
       </c>
-      <c r="B12" s="66"/>
-      <c r="C12" s="66"/>
-      <c r="D12" s="66"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
@@ -13741,7 +13709,7 @@
       <c r="B2" s="36"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="67" t="s">
+      <c r="A3" s="49" t="s">
         <v>393</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -13749,7 +13717,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="49" t="s">
         <v>395</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -13757,45 +13725,45 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="49" t="s">
         <v>397</v>
       </c>
-      <c r="B5" s="68" t="n">
+      <c r="B5" s="52" t="n">
         <v>4752655</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="67" t="s">
+      <c r="A6" s="49" t="s">
         <v>398</v>
       </c>
-      <c r="B6" s="68" t="n">
+      <c r="B6" s="52" t="n">
         <v>-1983194</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="49" t="s">
         <v>399</v>
       </c>
-      <c r="B7" s="68"/>
+      <c r="B7" s="52"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="67" t="s">
+      <c r="A8" s="49" t="s">
         <v>400</v>
       </c>
-      <c r="B8" s="68" t="n">
+      <c r="B8" s="52" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="67" t="s">
+      <c r="A9" s="49" t="s">
         <v>401</v>
       </c>
-      <c r="B9" s="68" t="n">
+      <c r="B9" s="52" t="n">
         <v>2770261</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="67" t="s">
+      <c r="A10" s="49" t="s">
         <v>402</v>
       </c>
       <c r="B10" s="1" t="n">
@@ -13804,7 +13772,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="67" t="s">
+      <c r="A11" s="49" t="s">
         <v>403</v>
       </c>
       <c r="B11" s="1" t="n">

</xml_diff>